<commit_message>
feat(fichas): corte en el I bimestre y escala vigesimal tentativa
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fichas/ficha_1_rendimiento.xlsx
+++ b/fichas/ficha_1_rendimiento.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Periodo de corte</t>
@@ -592,7 +592,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Datos acumulados hasta el cierre del I bimestre o I trimestre. El mismo corte se usa para el PRE 2026 y para el histórico 2024–2025, para que el modelo no aprenda de la ausencia de quien ya desertó.</t>
+          <t>Datos acumulados hasta el cierre del I bimestre. El mismo corte se usa para el PRE 2026 y para el histórico 2024–2025, para que el modelo no aprenda de la ausencia de quien ya desertó.</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,11 @@
           <t>Periodo de corte</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>I bimestre</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -7076,8 +7080,8 @@
       <formula1>2024</formula1>
       <formula2>2026</formula2>
     </dataValidation>
-    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija I bimestre o I trimestre." type="list">
-      <formula1>"I bimestre,I trimestre"</formula1>
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="El corte es el I bimestre." type="list">
+      <formula1>"I bimestre"</formula1>
     </dataValidation>
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una." type="list">
       <formula1>"vigesimal,literal"</formula1>

</xml_diff>

<commit_message>
feat(fichas): fichas pre-llenadas para rellenar y escala vigesimal
- generar_fichas.py --prellenar 2026_pre crea en data/raw/ las 3 fichas
  con los 70 códigos, grado, momento y año ya escritos y bloqueados
- D1 cerrada: escala vigesimal 0-20; se quita la escala literal
- preprocess.py informa los códigos sin usar en vez de contarlos como
  excluidos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fichas/ficha_1_rendimiento.xlsx
+++ b/fichas/ficha_1_rendimiento.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Datos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Conversión" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datos'!$A$9:$W$159</definedName>
@@ -24,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,10 +54,6 @@
     <font>
       <i val="1"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="6">
@@ -115,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,7 +143,6 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -532,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -652,60 +646,70 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Elija la escala en la celda B7. Con escala literal, AD/A/B/C se convierten según la hoja Conversión (provisional, decisión D1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Nota</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Una nota no válida para la escala elegida se marca en rojo y no se cuenta en el promedio.</t>
+          <t>Escala vigesimal (0 a 20), la que usa la IE. Se admiten decimales. Una nota fuera de 0-20 se marca en rojo y no se cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Diccionario de columnas (hoja Datos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Diccionario de columnas (hoja Datos)</t>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Columna</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Regla</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Columna</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Regla</t>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>codigo</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Código anonimizado del estudiante. Sin nombres ni DNI.</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>captura *</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Formato EST-### (ej. EST-001)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>grado</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Código anonimizado del estudiante. Sin nombres ni DNI.</t>
+          <t>Grado de secundaria.</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -715,19 +719,19 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Formato EST-### (ej. EST-001)</t>
+          <t>3 o 4</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>grado</t>
+          <t>seccion</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Grado de secundaria.</t>
+          <t>Sección (ej. A).</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -737,85 +741,85 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>3 o 4</t>
+          <t>1–2 caracteres</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>seccion</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Sección (ej. A).</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Grupo del diseño cuasiexperimental: 3.° = control, 4.° = experimental.</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>calculada</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Se calcula a partir del grado</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>momento</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Momento de la medición.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>captura *</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>1–2 caracteres</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>grupo</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Grupo del diseño cuasiexperimental: 3.° = control, 4.° = experimental.</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>calculada</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Se calcula a partir del grado</t>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>pre o post</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>momento</t>
+          <t>matematica</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Momento de la medición.</t>
+          <t>Nota final del I bimestre en Matemática (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>captura *</t>
+          <t>captura</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>pre o post</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>matematica</t>
+          <t>comunicacion</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Matemática. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Comunicación (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -825,19 +829,19 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>comunicacion</t>
+          <t>ingles</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Comunicación. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Inglés como lengua extranjera (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -847,19 +851,19 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>ingles</t>
+          <t>arte_cultura</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Inglés como lengua extranjera. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Arte y Cultura (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -869,19 +873,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>arte_cultura</t>
+          <t>ciencias_sociales</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Arte y Cultura. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Ciencias Sociales (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -891,19 +895,19 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>ciencias_sociales</t>
+          <t>dpcc</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Ciencias Sociales. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Desarrollo Personal, Ciudadanía y Cívica (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -913,19 +917,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>dpcc</t>
+          <t>educacion_fisica</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Desarrollo Personal, Ciudadanía y Cívica. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Educación Física (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -935,19 +939,19 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>educacion_fisica</t>
+          <t>educacion_religiosa</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Educación Física. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Educación Religiosa (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -957,19 +961,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>educacion_religiosa</t>
+          <t>ciencia_tecnologia</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Educación Religiosa. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Ciencia y Tecnología (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -979,19 +983,19 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>ciencia_tecnologia</t>
+          <t>ept</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Calificación del periodo en Ciencia y Tecnología. Vacío si no aplica (ej. exonerado).</t>
+          <t>Nota final del I bimestre en Educación para el Trabajo (0 a 20). Vacío si no aplica (ej. exonerado).</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -1001,41 +1005,41 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+          <t>0 a 20</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>ept</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Calificación del periodo en Educación para el Trabajo. Vacío si no aplica (ej. exonerado).</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>captura</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>0–20 (vigesimal) o AD/A/B/C (literal)</t>
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>n_notas</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>n: cantidad de calificaciones válidas registradas.</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>calculada</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Cuenta solo notas válidas</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>n_notas</t>
+          <t>suma_notas</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>n: cantidad de calificaciones válidas registradas.</t>
+          <t>Σ Notas.</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -1045,19 +1049,19 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Cuenta solo notas válidas</t>
+          <t>Σ Notas</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>suma_notas</t>
+          <t>promedio</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Σ Notas. En escala literal suma los valores de la hoja Conversión.</t>
+          <t>Promedio = Σ Notas / n, redondeado a 2 decimales.</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -1067,63 +1071,63 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Σ Notas</t>
+          <t>Σ Notas / n</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>promedio</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Promedio = Σ Notas / n, redondeado a 2 decimales.</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>calculada</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Σ Notas / n</t>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>anio</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Año lectivo del registro. 2024–2025 = histórico de entrenamiento.</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>captura *</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>2024, 2025 o 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>anio</t>
+          <t>deserto</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Año lectivo del registro. 2024–2025 = histórico de entrenamiento.</t>
+          <t>Solo histórico 2024–2025: 1 si abandonó ese año, 0 si no. Dejar vacío en 2026.</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>captura *</t>
+          <t>captura</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>2024, 2025 o 2026</t>
+          <t>0 o 1; vacío en 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>deserto</t>
+          <t>excluido</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Solo histórico 2024–2025: 1 si abandonó ese año, 0 si no. Dejar vacío en 2026.</t>
+          <t>Marcar sí si cumple un criterio de exclusión de la tesis.</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -1133,19 +1137,19 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>0 o 1; vacío en 2026</t>
+          <t>sí o no</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>excluido</t>
+          <t>motivo_exclusion</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Marcar sí si cumple un criterio de exclusión de la tesis.</t>
+          <t>Obligatorio si excluido = sí.</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -1155,19 +1159,19 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>sí o no</t>
+          <t>traslado definitivo / dimensión incompleta / registro inconsistente</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>motivo_exclusion</t>
+          <t>observaciones</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Obligatorio si excluido = sí.</t>
+          <t>Texto libre (sin datos personales).</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -1175,39 +1179,17 @@
           <t>captura</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>traslado definitivo / dimensión incompleta / registro inconsistente</t>
-        </is>
-      </c>
+      <c r="D37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>observaciones</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Texto libre (sin datos personales).</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>captura</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>* obligatoria</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B3:D3"/>
@@ -1215,7 +1197,6 @@
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B12:D12"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B6:D6"/>
   </mergeCells>
@@ -1313,18 +1294,6 @@
       </c>
       <c r="B6" s="10" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Escala de calificación</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>vigesimal</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -1462,11 +1431,11 @@
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="n"/>
       <c r="P10" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F10:O10,'Conversión'!$A$5:$A$8)),COUNTIFS(F10:O10,"&gt;=0",F10:O10,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F10:O10,'Conversión'!$A$5:$A$8)),COUNTIFS(F10:O10,"&gt;=0",F10:O10,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F10:O10,"&gt;=0",F10:O10,"&lt;=20")=0,"",COUNTIFS(F10:O10,"&gt;=0",F10:O10,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q10" s="15">
-        <f>IF(P10="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F10:O10,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F10:O10,F10:O10,"&gt;=0",F10:O10,"&lt;=20")))</f>
+        <f>IF(P10="","",SUMIFS(F10:O10,F10:O10,"&gt;=0",F10:O10,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R10" s="15">
@@ -1499,11 +1468,11 @@
       <c r="N11" s="14" t="n"/>
       <c r="O11" s="14" t="n"/>
       <c r="P11" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F11:O11,'Conversión'!$A$5:$A$8)),COUNTIFS(F11:O11,"&gt;=0",F11:O11,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F11:O11,'Conversión'!$A$5:$A$8)),COUNTIFS(F11:O11,"&gt;=0",F11:O11,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F11:O11,"&gt;=0",F11:O11,"&lt;=20")=0,"",COUNTIFS(F11:O11,"&gt;=0",F11:O11,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q11" s="15">
-        <f>IF(P11="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F11:O11,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F11:O11,F11:O11,"&gt;=0",F11:O11,"&lt;=20")))</f>
+        <f>IF(P11="","",SUMIFS(F11:O11,F11:O11,"&gt;=0",F11:O11,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R11" s="15">
@@ -1536,11 +1505,11 @@
       <c r="N12" s="14" t="n"/>
       <c r="O12" s="14" t="n"/>
       <c r="P12" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F12:O12,'Conversión'!$A$5:$A$8)),COUNTIFS(F12:O12,"&gt;=0",F12:O12,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F12:O12,'Conversión'!$A$5:$A$8)),COUNTIFS(F12:O12,"&gt;=0",F12:O12,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F12:O12,"&gt;=0",F12:O12,"&lt;=20")=0,"",COUNTIFS(F12:O12,"&gt;=0",F12:O12,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q12" s="15">
-        <f>IF(P12="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F12:O12,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F12:O12,F12:O12,"&gt;=0",F12:O12,"&lt;=20")))</f>
+        <f>IF(P12="","",SUMIFS(F12:O12,F12:O12,"&gt;=0",F12:O12,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R12" s="15">
@@ -1573,11 +1542,11 @@
       <c r="N13" s="14" t="n"/>
       <c r="O13" s="14" t="n"/>
       <c r="P13" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F13:O13,'Conversión'!$A$5:$A$8)),COUNTIFS(F13:O13,"&gt;=0",F13:O13,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F13:O13,'Conversión'!$A$5:$A$8)),COUNTIFS(F13:O13,"&gt;=0",F13:O13,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F13:O13,"&gt;=0",F13:O13,"&lt;=20")=0,"",COUNTIFS(F13:O13,"&gt;=0",F13:O13,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q13" s="15">
-        <f>IF(P13="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F13:O13,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F13:O13,F13:O13,"&gt;=0",F13:O13,"&lt;=20")))</f>
+        <f>IF(P13="","",SUMIFS(F13:O13,F13:O13,"&gt;=0",F13:O13,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R13" s="15">
@@ -1610,11 +1579,11 @@
       <c r="N14" s="14" t="n"/>
       <c r="O14" s="14" t="n"/>
       <c r="P14" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F14:O14,'Conversión'!$A$5:$A$8)),COUNTIFS(F14:O14,"&gt;=0",F14:O14,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F14:O14,'Conversión'!$A$5:$A$8)),COUNTIFS(F14:O14,"&gt;=0",F14:O14,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F14:O14,"&gt;=0",F14:O14,"&lt;=20")=0,"",COUNTIFS(F14:O14,"&gt;=0",F14:O14,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q14" s="15">
-        <f>IF(P14="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F14:O14,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F14:O14,F14:O14,"&gt;=0",F14:O14,"&lt;=20")))</f>
+        <f>IF(P14="","",SUMIFS(F14:O14,F14:O14,"&gt;=0",F14:O14,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R14" s="15">
@@ -1647,11 +1616,11 @@
       <c r="N15" s="14" t="n"/>
       <c r="O15" s="14" t="n"/>
       <c r="P15" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F15:O15,'Conversión'!$A$5:$A$8)),COUNTIFS(F15:O15,"&gt;=0",F15:O15,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F15:O15,'Conversión'!$A$5:$A$8)),COUNTIFS(F15:O15,"&gt;=0",F15:O15,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F15:O15,"&gt;=0",F15:O15,"&lt;=20")=0,"",COUNTIFS(F15:O15,"&gt;=0",F15:O15,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q15" s="15">
-        <f>IF(P15="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F15:O15,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F15:O15,F15:O15,"&gt;=0",F15:O15,"&lt;=20")))</f>
+        <f>IF(P15="","",SUMIFS(F15:O15,F15:O15,"&gt;=0",F15:O15,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R15" s="15">
@@ -1684,11 +1653,11 @@
       <c r="N16" s="14" t="n"/>
       <c r="O16" s="14" t="n"/>
       <c r="P16" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F16:O16,'Conversión'!$A$5:$A$8)),COUNTIFS(F16:O16,"&gt;=0",F16:O16,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F16:O16,'Conversión'!$A$5:$A$8)),COUNTIFS(F16:O16,"&gt;=0",F16:O16,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F16:O16,"&gt;=0",F16:O16,"&lt;=20")=0,"",COUNTIFS(F16:O16,"&gt;=0",F16:O16,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q16" s="15">
-        <f>IF(P16="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F16:O16,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F16:O16,F16:O16,"&gt;=0",F16:O16,"&lt;=20")))</f>
+        <f>IF(P16="","",SUMIFS(F16:O16,F16:O16,"&gt;=0",F16:O16,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R16" s="15">
@@ -1721,11 +1690,11 @@
       <c r="N17" s="14" t="n"/>
       <c r="O17" s="14" t="n"/>
       <c r="P17" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F17:O17,'Conversión'!$A$5:$A$8)),COUNTIFS(F17:O17,"&gt;=0",F17:O17,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F17:O17,'Conversión'!$A$5:$A$8)),COUNTIFS(F17:O17,"&gt;=0",F17:O17,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F17:O17,"&gt;=0",F17:O17,"&lt;=20")=0,"",COUNTIFS(F17:O17,"&gt;=0",F17:O17,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q17" s="15">
-        <f>IF(P17="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F17:O17,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F17:O17,F17:O17,"&gt;=0",F17:O17,"&lt;=20")))</f>
+        <f>IF(P17="","",SUMIFS(F17:O17,F17:O17,"&gt;=0",F17:O17,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R17" s="15">
@@ -1758,11 +1727,11 @@
       <c r="N18" s="14" t="n"/>
       <c r="O18" s="14" t="n"/>
       <c r="P18" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F18:O18,'Conversión'!$A$5:$A$8)),COUNTIFS(F18:O18,"&gt;=0",F18:O18,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F18:O18,'Conversión'!$A$5:$A$8)),COUNTIFS(F18:O18,"&gt;=0",F18:O18,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F18:O18,"&gt;=0",F18:O18,"&lt;=20")=0,"",COUNTIFS(F18:O18,"&gt;=0",F18:O18,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q18" s="15">
-        <f>IF(P18="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F18:O18,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F18:O18,F18:O18,"&gt;=0",F18:O18,"&lt;=20")))</f>
+        <f>IF(P18="","",SUMIFS(F18:O18,F18:O18,"&gt;=0",F18:O18,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R18" s="15">
@@ -1795,11 +1764,11 @@
       <c r="N19" s="14" t="n"/>
       <c r="O19" s="14" t="n"/>
       <c r="P19" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F19:O19,'Conversión'!$A$5:$A$8)),COUNTIFS(F19:O19,"&gt;=0",F19:O19,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F19:O19,'Conversión'!$A$5:$A$8)),COUNTIFS(F19:O19,"&gt;=0",F19:O19,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F19:O19,"&gt;=0",F19:O19,"&lt;=20")=0,"",COUNTIFS(F19:O19,"&gt;=0",F19:O19,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q19" s="15">
-        <f>IF(P19="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F19:O19,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F19:O19,F19:O19,"&gt;=0",F19:O19,"&lt;=20")))</f>
+        <f>IF(P19="","",SUMIFS(F19:O19,F19:O19,"&gt;=0",F19:O19,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R19" s="15">
@@ -1832,11 +1801,11 @@
       <c r="N20" s="14" t="n"/>
       <c r="O20" s="14" t="n"/>
       <c r="P20" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F20:O20,'Conversión'!$A$5:$A$8)),COUNTIFS(F20:O20,"&gt;=0",F20:O20,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F20:O20,'Conversión'!$A$5:$A$8)),COUNTIFS(F20:O20,"&gt;=0",F20:O20,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F20:O20,"&gt;=0",F20:O20,"&lt;=20")=0,"",COUNTIFS(F20:O20,"&gt;=0",F20:O20,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q20" s="15">
-        <f>IF(P20="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F20:O20,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F20:O20,F20:O20,"&gt;=0",F20:O20,"&lt;=20")))</f>
+        <f>IF(P20="","",SUMIFS(F20:O20,F20:O20,"&gt;=0",F20:O20,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R20" s="15">
@@ -1869,11 +1838,11 @@
       <c r="N21" s="14" t="n"/>
       <c r="O21" s="14" t="n"/>
       <c r="P21" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F21:O21,'Conversión'!$A$5:$A$8)),COUNTIFS(F21:O21,"&gt;=0",F21:O21,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F21:O21,'Conversión'!$A$5:$A$8)),COUNTIFS(F21:O21,"&gt;=0",F21:O21,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F21:O21,"&gt;=0",F21:O21,"&lt;=20")=0,"",COUNTIFS(F21:O21,"&gt;=0",F21:O21,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q21" s="15">
-        <f>IF(P21="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F21:O21,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F21:O21,F21:O21,"&gt;=0",F21:O21,"&lt;=20")))</f>
+        <f>IF(P21="","",SUMIFS(F21:O21,F21:O21,"&gt;=0",F21:O21,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R21" s="15">
@@ -1906,11 +1875,11 @@
       <c r="N22" s="14" t="n"/>
       <c r="O22" s="14" t="n"/>
       <c r="P22" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F22:O22,'Conversión'!$A$5:$A$8)),COUNTIFS(F22:O22,"&gt;=0",F22:O22,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F22:O22,'Conversión'!$A$5:$A$8)),COUNTIFS(F22:O22,"&gt;=0",F22:O22,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F22:O22,"&gt;=0",F22:O22,"&lt;=20")=0,"",COUNTIFS(F22:O22,"&gt;=0",F22:O22,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q22" s="15">
-        <f>IF(P22="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F22:O22,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F22:O22,F22:O22,"&gt;=0",F22:O22,"&lt;=20")))</f>
+        <f>IF(P22="","",SUMIFS(F22:O22,F22:O22,"&gt;=0",F22:O22,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R22" s="15">
@@ -1943,11 +1912,11 @@
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="14" t="n"/>
       <c r="P23" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F23:O23,'Conversión'!$A$5:$A$8)),COUNTIFS(F23:O23,"&gt;=0",F23:O23,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F23:O23,'Conversión'!$A$5:$A$8)),COUNTIFS(F23:O23,"&gt;=0",F23:O23,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F23:O23,"&gt;=0",F23:O23,"&lt;=20")=0,"",COUNTIFS(F23:O23,"&gt;=0",F23:O23,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q23" s="15">
-        <f>IF(P23="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F23:O23,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F23:O23,F23:O23,"&gt;=0",F23:O23,"&lt;=20")))</f>
+        <f>IF(P23="","",SUMIFS(F23:O23,F23:O23,"&gt;=0",F23:O23,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R23" s="15">
@@ -1980,11 +1949,11 @@
       <c r="N24" s="14" t="n"/>
       <c r="O24" s="14" t="n"/>
       <c r="P24" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F24:O24,'Conversión'!$A$5:$A$8)),COUNTIFS(F24:O24,"&gt;=0",F24:O24,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F24:O24,'Conversión'!$A$5:$A$8)),COUNTIFS(F24:O24,"&gt;=0",F24:O24,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F24:O24,"&gt;=0",F24:O24,"&lt;=20")=0,"",COUNTIFS(F24:O24,"&gt;=0",F24:O24,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q24" s="15">
-        <f>IF(P24="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F24:O24,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F24:O24,F24:O24,"&gt;=0",F24:O24,"&lt;=20")))</f>
+        <f>IF(P24="","",SUMIFS(F24:O24,F24:O24,"&gt;=0",F24:O24,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R24" s="15">
@@ -2017,11 +1986,11 @@
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="14" t="n"/>
       <c r="P25" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F25:O25,'Conversión'!$A$5:$A$8)),COUNTIFS(F25:O25,"&gt;=0",F25:O25,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F25:O25,'Conversión'!$A$5:$A$8)),COUNTIFS(F25:O25,"&gt;=0",F25:O25,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F25:O25,"&gt;=0",F25:O25,"&lt;=20")=0,"",COUNTIFS(F25:O25,"&gt;=0",F25:O25,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q25" s="15">
-        <f>IF(P25="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F25:O25,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F25:O25,F25:O25,"&gt;=0",F25:O25,"&lt;=20")))</f>
+        <f>IF(P25="","",SUMIFS(F25:O25,F25:O25,"&gt;=0",F25:O25,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R25" s="15">
@@ -2054,11 +2023,11 @@
       <c r="N26" s="14" t="n"/>
       <c r="O26" s="14" t="n"/>
       <c r="P26" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F26:O26,'Conversión'!$A$5:$A$8)),COUNTIFS(F26:O26,"&gt;=0",F26:O26,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F26:O26,'Conversión'!$A$5:$A$8)),COUNTIFS(F26:O26,"&gt;=0",F26:O26,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F26:O26,"&gt;=0",F26:O26,"&lt;=20")=0,"",COUNTIFS(F26:O26,"&gt;=0",F26:O26,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q26" s="15">
-        <f>IF(P26="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F26:O26,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F26:O26,F26:O26,"&gt;=0",F26:O26,"&lt;=20")))</f>
+        <f>IF(P26="","",SUMIFS(F26:O26,F26:O26,"&gt;=0",F26:O26,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R26" s="15">
@@ -2091,11 +2060,11 @@
       <c r="N27" s="14" t="n"/>
       <c r="O27" s="14" t="n"/>
       <c r="P27" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F27:O27,'Conversión'!$A$5:$A$8)),COUNTIFS(F27:O27,"&gt;=0",F27:O27,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F27:O27,'Conversión'!$A$5:$A$8)),COUNTIFS(F27:O27,"&gt;=0",F27:O27,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F27:O27,"&gt;=0",F27:O27,"&lt;=20")=0,"",COUNTIFS(F27:O27,"&gt;=0",F27:O27,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q27" s="15">
-        <f>IF(P27="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F27:O27,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F27:O27,F27:O27,"&gt;=0",F27:O27,"&lt;=20")))</f>
+        <f>IF(P27="","",SUMIFS(F27:O27,F27:O27,"&gt;=0",F27:O27,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R27" s="15">
@@ -2128,11 +2097,11 @@
       <c r="N28" s="14" t="n"/>
       <c r="O28" s="14" t="n"/>
       <c r="P28" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F28:O28,'Conversión'!$A$5:$A$8)),COUNTIFS(F28:O28,"&gt;=0",F28:O28,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F28:O28,'Conversión'!$A$5:$A$8)),COUNTIFS(F28:O28,"&gt;=0",F28:O28,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F28:O28,"&gt;=0",F28:O28,"&lt;=20")=0,"",COUNTIFS(F28:O28,"&gt;=0",F28:O28,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q28" s="15">
-        <f>IF(P28="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F28:O28,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F28:O28,F28:O28,"&gt;=0",F28:O28,"&lt;=20")))</f>
+        <f>IF(P28="","",SUMIFS(F28:O28,F28:O28,"&gt;=0",F28:O28,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R28" s="15">
@@ -2165,11 +2134,11 @@
       <c r="N29" s="14" t="n"/>
       <c r="O29" s="14" t="n"/>
       <c r="P29" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F29:O29,'Conversión'!$A$5:$A$8)),COUNTIFS(F29:O29,"&gt;=0",F29:O29,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F29:O29,'Conversión'!$A$5:$A$8)),COUNTIFS(F29:O29,"&gt;=0",F29:O29,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F29:O29,"&gt;=0",F29:O29,"&lt;=20")=0,"",COUNTIFS(F29:O29,"&gt;=0",F29:O29,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q29" s="15">
-        <f>IF(P29="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F29:O29,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F29:O29,F29:O29,"&gt;=0",F29:O29,"&lt;=20")))</f>
+        <f>IF(P29="","",SUMIFS(F29:O29,F29:O29,"&gt;=0",F29:O29,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R29" s="15">
@@ -2202,11 +2171,11 @@
       <c r="N30" s="14" t="n"/>
       <c r="O30" s="14" t="n"/>
       <c r="P30" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F30:O30,'Conversión'!$A$5:$A$8)),COUNTIFS(F30:O30,"&gt;=0",F30:O30,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F30:O30,'Conversión'!$A$5:$A$8)),COUNTIFS(F30:O30,"&gt;=0",F30:O30,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F30:O30,"&gt;=0",F30:O30,"&lt;=20")=0,"",COUNTIFS(F30:O30,"&gt;=0",F30:O30,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q30" s="15">
-        <f>IF(P30="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F30:O30,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F30:O30,F30:O30,"&gt;=0",F30:O30,"&lt;=20")))</f>
+        <f>IF(P30="","",SUMIFS(F30:O30,F30:O30,"&gt;=0",F30:O30,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R30" s="15">
@@ -2239,11 +2208,11 @@
       <c r="N31" s="14" t="n"/>
       <c r="O31" s="14" t="n"/>
       <c r="P31" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F31:O31,'Conversión'!$A$5:$A$8)),COUNTIFS(F31:O31,"&gt;=0",F31:O31,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F31:O31,'Conversión'!$A$5:$A$8)),COUNTIFS(F31:O31,"&gt;=0",F31:O31,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F31:O31,"&gt;=0",F31:O31,"&lt;=20")=0,"",COUNTIFS(F31:O31,"&gt;=0",F31:O31,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q31" s="15">
-        <f>IF(P31="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F31:O31,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F31:O31,F31:O31,"&gt;=0",F31:O31,"&lt;=20")))</f>
+        <f>IF(P31="","",SUMIFS(F31:O31,F31:O31,"&gt;=0",F31:O31,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R31" s="15">
@@ -2276,11 +2245,11 @@
       <c r="N32" s="14" t="n"/>
       <c r="O32" s="14" t="n"/>
       <c r="P32" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F32:O32,'Conversión'!$A$5:$A$8)),COUNTIFS(F32:O32,"&gt;=0",F32:O32,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F32:O32,'Conversión'!$A$5:$A$8)),COUNTIFS(F32:O32,"&gt;=0",F32:O32,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F32:O32,"&gt;=0",F32:O32,"&lt;=20")=0,"",COUNTIFS(F32:O32,"&gt;=0",F32:O32,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q32" s="15">
-        <f>IF(P32="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F32:O32,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F32:O32,F32:O32,"&gt;=0",F32:O32,"&lt;=20")))</f>
+        <f>IF(P32="","",SUMIFS(F32:O32,F32:O32,"&gt;=0",F32:O32,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R32" s="15">
@@ -2313,11 +2282,11 @@
       <c r="N33" s="14" t="n"/>
       <c r="O33" s="14" t="n"/>
       <c r="P33" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F33:O33,'Conversión'!$A$5:$A$8)),COUNTIFS(F33:O33,"&gt;=0",F33:O33,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F33:O33,'Conversión'!$A$5:$A$8)),COUNTIFS(F33:O33,"&gt;=0",F33:O33,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F33:O33,"&gt;=0",F33:O33,"&lt;=20")=0,"",COUNTIFS(F33:O33,"&gt;=0",F33:O33,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q33" s="15">
-        <f>IF(P33="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F33:O33,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F33:O33,F33:O33,"&gt;=0",F33:O33,"&lt;=20")))</f>
+        <f>IF(P33="","",SUMIFS(F33:O33,F33:O33,"&gt;=0",F33:O33,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R33" s="15">
@@ -2350,11 +2319,11 @@
       <c r="N34" s="14" t="n"/>
       <c r="O34" s="14" t="n"/>
       <c r="P34" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F34:O34,'Conversión'!$A$5:$A$8)),COUNTIFS(F34:O34,"&gt;=0",F34:O34,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F34:O34,'Conversión'!$A$5:$A$8)),COUNTIFS(F34:O34,"&gt;=0",F34:O34,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F34:O34,"&gt;=0",F34:O34,"&lt;=20")=0,"",COUNTIFS(F34:O34,"&gt;=0",F34:O34,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q34" s="15">
-        <f>IF(P34="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F34:O34,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F34:O34,F34:O34,"&gt;=0",F34:O34,"&lt;=20")))</f>
+        <f>IF(P34="","",SUMIFS(F34:O34,F34:O34,"&gt;=0",F34:O34,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R34" s="15">
@@ -2387,11 +2356,11 @@
       <c r="N35" s="14" t="n"/>
       <c r="O35" s="14" t="n"/>
       <c r="P35" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F35:O35,'Conversión'!$A$5:$A$8)),COUNTIFS(F35:O35,"&gt;=0",F35:O35,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F35:O35,'Conversión'!$A$5:$A$8)),COUNTIFS(F35:O35,"&gt;=0",F35:O35,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F35:O35,"&gt;=0",F35:O35,"&lt;=20")=0,"",COUNTIFS(F35:O35,"&gt;=0",F35:O35,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q35" s="15">
-        <f>IF(P35="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F35:O35,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F35:O35,F35:O35,"&gt;=0",F35:O35,"&lt;=20")))</f>
+        <f>IF(P35="","",SUMIFS(F35:O35,F35:O35,"&gt;=0",F35:O35,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R35" s="15">
@@ -2424,11 +2393,11 @@
       <c r="N36" s="14" t="n"/>
       <c r="O36" s="14" t="n"/>
       <c r="P36" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F36:O36,'Conversión'!$A$5:$A$8)),COUNTIFS(F36:O36,"&gt;=0",F36:O36,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F36:O36,'Conversión'!$A$5:$A$8)),COUNTIFS(F36:O36,"&gt;=0",F36:O36,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F36:O36,"&gt;=0",F36:O36,"&lt;=20")=0,"",COUNTIFS(F36:O36,"&gt;=0",F36:O36,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q36" s="15">
-        <f>IF(P36="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F36:O36,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F36:O36,F36:O36,"&gt;=0",F36:O36,"&lt;=20")))</f>
+        <f>IF(P36="","",SUMIFS(F36:O36,F36:O36,"&gt;=0",F36:O36,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R36" s="15">
@@ -2461,11 +2430,11 @@
       <c r="N37" s="14" t="n"/>
       <c r="O37" s="14" t="n"/>
       <c r="P37" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F37:O37,'Conversión'!$A$5:$A$8)),COUNTIFS(F37:O37,"&gt;=0",F37:O37,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F37:O37,'Conversión'!$A$5:$A$8)),COUNTIFS(F37:O37,"&gt;=0",F37:O37,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F37:O37,"&gt;=0",F37:O37,"&lt;=20")=0,"",COUNTIFS(F37:O37,"&gt;=0",F37:O37,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q37" s="15">
-        <f>IF(P37="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F37:O37,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F37:O37,F37:O37,"&gt;=0",F37:O37,"&lt;=20")))</f>
+        <f>IF(P37="","",SUMIFS(F37:O37,F37:O37,"&gt;=0",F37:O37,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R37" s="15">
@@ -2498,11 +2467,11 @@
       <c r="N38" s="14" t="n"/>
       <c r="O38" s="14" t="n"/>
       <c r="P38" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F38:O38,'Conversión'!$A$5:$A$8)),COUNTIFS(F38:O38,"&gt;=0",F38:O38,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F38:O38,'Conversión'!$A$5:$A$8)),COUNTIFS(F38:O38,"&gt;=0",F38:O38,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F38:O38,"&gt;=0",F38:O38,"&lt;=20")=0,"",COUNTIFS(F38:O38,"&gt;=0",F38:O38,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q38" s="15">
-        <f>IF(P38="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F38:O38,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F38:O38,F38:O38,"&gt;=0",F38:O38,"&lt;=20")))</f>
+        <f>IF(P38="","",SUMIFS(F38:O38,F38:O38,"&gt;=0",F38:O38,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R38" s="15">
@@ -2535,11 +2504,11 @@
       <c r="N39" s="14" t="n"/>
       <c r="O39" s="14" t="n"/>
       <c r="P39" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F39:O39,'Conversión'!$A$5:$A$8)),COUNTIFS(F39:O39,"&gt;=0",F39:O39,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F39:O39,'Conversión'!$A$5:$A$8)),COUNTIFS(F39:O39,"&gt;=0",F39:O39,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F39:O39,"&gt;=0",F39:O39,"&lt;=20")=0,"",COUNTIFS(F39:O39,"&gt;=0",F39:O39,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q39" s="15">
-        <f>IF(P39="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F39:O39,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F39:O39,F39:O39,"&gt;=0",F39:O39,"&lt;=20")))</f>
+        <f>IF(P39="","",SUMIFS(F39:O39,F39:O39,"&gt;=0",F39:O39,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R39" s="15">
@@ -2572,11 +2541,11 @@
       <c r="N40" s="14" t="n"/>
       <c r="O40" s="14" t="n"/>
       <c r="P40" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F40:O40,'Conversión'!$A$5:$A$8)),COUNTIFS(F40:O40,"&gt;=0",F40:O40,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F40:O40,'Conversión'!$A$5:$A$8)),COUNTIFS(F40:O40,"&gt;=0",F40:O40,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F40:O40,"&gt;=0",F40:O40,"&lt;=20")=0,"",COUNTIFS(F40:O40,"&gt;=0",F40:O40,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q40" s="15">
-        <f>IF(P40="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F40:O40,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F40:O40,F40:O40,"&gt;=0",F40:O40,"&lt;=20")))</f>
+        <f>IF(P40="","",SUMIFS(F40:O40,F40:O40,"&gt;=0",F40:O40,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R40" s="15">
@@ -2609,11 +2578,11 @@
       <c r="N41" s="14" t="n"/>
       <c r="O41" s="14" t="n"/>
       <c r="P41" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F41:O41,'Conversión'!$A$5:$A$8)),COUNTIFS(F41:O41,"&gt;=0",F41:O41,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F41:O41,'Conversión'!$A$5:$A$8)),COUNTIFS(F41:O41,"&gt;=0",F41:O41,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F41:O41,"&gt;=0",F41:O41,"&lt;=20")=0,"",COUNTIFS(F41:O41,"&gt;=0",F41:O41,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q41" s="15">
-        <f>IF(P41="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F41:O41,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F41:O41,F41:O41,"&gt;=0",F41:O41,"&lt;=20")))</f>
+        <f>IF(P41="","",SUMIFS(F41:O41,F41:O41,"&gt;=0",F41:O41,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R41" s="15">
@@ -2646,11 +2615,11 @@
       <c r="N42" s="14" t="n"/>
       <c r="O42" s="14" t="n"/>
       <c r="P42" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F42:O42,'Conversión'!$A$5:$A$8)),COUNTIFS(F42:O42,"&gt;=0",F42:O42,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F42:O42,'Conversión'!$A$5:$A$8)),COUNTIFS(F42:O42,"&gt;=0",F42:O42,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F42:O42,"&gt;=0",F42:O42,"&lt;=20")=0,"",COUNTIFS(F42:O42,"&gt;=0",F42:O42,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q42" s="15">
-        <f>IF(P42="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F42:O42,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F42:O42,F42:O42,"&gt;=0",F42:O42,"&lt;=20")))</f>
+        <f>IF(P42="","",SUMIFS(F42:O42,F42:O42,"&gt;=0",F42:O42,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R42" s="15">
@@ -2683,11 +2652,11 @@
       <c r="N43" s="14" t="n"/>
       <c r="O43" s="14" t="n"/>
       <c r="P43" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F43:O43,'Conversión'!$A$5:$A$8)),COUNTIFS(F43:O43,"&gt;=0",F43:O43,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F43:O43,'Conversión'!$A$5:$A$8)),COUNTIFS(F43:O43,"&gt;=0",F43:O43,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F43:O43,"&gt;=0",F43:O43,"&lt;=20")=0,"",COUNTIFS(F43:O43,"&gt;=0",F43:O43,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q43" s="15">
-        <f>IF(P43="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F43:O43,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F43:O43,F43:O43,"&gt;=0",F43:O43,"&lt;=20")))</f>
+        <f>IF(P43="","",SUMIFS(F43:O43,F43:O43,"&gt;=0",F43:O43,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R43" s="15">
@@ -2720,11 +2689,11 @@
       <c r="N44" s="14" t="n"/>
       <c r="O44" s="14" t="n"/>
       <c r="P44" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F44:O44,'Conversión'!$A$5:$A$8)),COUNTIFS(F44:O44,"&gt;=0",F44:O44,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F44:O44,'Conversión'!$A$5:$A$8)),COUNTIFS(F44:O44,"&gt;=0",F44:O44,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F44:O44,"&gt;=0",F44:O44,"&lt;=20")=0,"",COUNTIFS(F44:O44,"&gt;=0",F44:O44,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q44" s="15">
-        <f>IF(P44="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F44:O44,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F44:O44,F44:O44,"&gt;=0",F44:O44,"&lt;=20")))</f>
+        <f>IF(P44="","",SUMIFS(F44:O44,F44:O44,"&gt;=0",F44:O44,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R44" s="15">
@@ -2757,11 +2726,11 @@
       <c r="N45" s="14" t="n"/>
       <c r="O45" s="14" t="n"/>
       <c r="P45" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F45:O45,'Conversión'!$A$5:$A$8)),COUNTIFS(F45:O45,"&gt;=0",F45:O45,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F45:O45,'Conversión'!$A$5:$A$8)),COUNTIFS(F45:O45,"&gt;=0",F45:O45,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F45:O45,"&gt;=0",F45:O45,"&lt;=20")=0,"",COUNTIFS(F45:O45,"&gt;=0",F45:O45,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q45" s="15">
-        <f>IF(P45="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F45:O45,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F45:O45,F45:O45,"&gt;=0",F45:O45,"&lt;=20")))</f>
+        <f>IF(P45="","",SUMIFS(F45:O45,F45:O45,"&gt;=0",F45:O45,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R45" s="15">
@@ -2794,11 +2763,11 @@
       <c r="N46" s="14" t="n"/>
       <c r="O46" s="14" t="n"/>
       <c r="P46" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F46:O46,'Conversión'!$A$5:$A$8)),COUNTIFS(F46:O46,"&gt;=0",F46:O46,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F46:O46,'Conversión'!$A$5:$A$8)),COUNTIFS(F46:O46,"&gt;=0",F46:O46,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F46:O46,"&gt;=0",F46:O46,"&lt;=20")=0,"",COUNTIFS(F46:O46,"&gt;=0",F46:O46,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q46" s="15">
-        <f>IF(P46="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F46:O46,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F46:O46,F46:O46,"&gt;=0",F46:O46,"&lt;=20")))</f>
+        <f>IF(P46="","",SUMIFS(F46:O46,F46:O46,"&gt;=0",F46:O46,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R46" s="15">
@@ -2831,11 +2800,11 @@
       <c r="N47" s="14" t="n"/>
       <c r="O47" s="14" t="n"/>
       <c r="P47" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F47:O47,'Conversión'!$A$5:$A$8)),COUNTIFS(F47:O47,"&gt;=0",F47:O47,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F47:O47,'Conversión'!$A$5:$A$8)),COUNTIFS(F47:O47,"&gt;=0",F47:O47,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F47:O47,"&gt;=0",F47:O47,"&lt;=20")=0,"",COUNTIFS(F47:O47,"&gt;=0",F47:O47,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q47" s="15">
-        <f>IF(P47="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F47:O47,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F47:O47,F47:O47,"&gt;=0",F47:O47,"&lt;=20")))</f>
+        <f>IF(P47="","",SUMIFS(F47:O47,F47:O47,"&gt;=0",F47:O47,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R47" s="15">
@@ -2868,11 +2837,11 @@
       <c r="N48" s="14" t="n"/>
       <c r="O48" s="14" t="n"/>
       <c r="P48" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F48:O48,'Conversión'!$A$5:$A$8)),COUNTIFS(F48:O48,"&gt;=0",F48:O48,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F48:O48,'Conversión'!$A$5:$A$8)),COUNTIFS(F48:O48,"&gt;=0",F48:O48,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F48:O48,"&gt;=0",F48:O48,"&lt;=20")=0,"",COUNTIFS(F48:O48,"&gt;=0",F48:O48,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q48" s="15">
-        <f>IF(P48="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F48:O48,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F48:O48,F48:O48,"&gt;=0",F48:O48,"&lt;=20")))</f>
+        <f>IF(P48="","",SUMIFS(F48:O48,F48:O48,"&gt;=0",F48:O48,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R48" s="15">
@@ -2905,11 +2874,11 @@
       <c r="N49" s="14" t="n"/>
       <c r="O49" s="14" t="n"/>
       <c r="P49" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F49:O49,'Conversión'!$A$5:$A$8)),COUNTIFS(F49:O49,"&gt;=0",F49:O49,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F49:O49,'Conversión'!$A$5:$A$8)),COUNTIFS(F49:O49,"&gt;=0",F49:O49,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F49:O49,"&gt;=0",F49:O49,"&lt;=20")=0,"",COUNTIFS(F49:O49,"&gt;=0",F49:O49,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q49" s="15">
-        <f>IF(P49="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F49:O49,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F49:O49,F49:O49,"&gt;=0",F49:O49,"&lt;=20")))</f>
+        <f>IF(P49="","",SUMIFS(F49:O49,F49:O49,"&gt;=0",F49:O49,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R49" s="15">
@@ -2942,11 +2911,11 @@
       <c r="N50" s="14" t="n"/>
       <c r="O50" s="14" t="n"/>
       <c r="P50" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F50:O50,'Conversión'!$A$5:$A$8)),COUNTIFS(F50:O50,"&gt;=0",F50:O50,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F50:O50,'Conversión'!$A$5:$A$8)),COUNTIFS(F50:O50,"&gt;=0",F50:O50,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F50:O50,"&gt;=0",F50:O50,"&lt;=20")=0,"",COUNTIFS(F50:O50,"&gt;=0",F50:O50,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q50" s="15">
-        <f>IF(P50="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F50:O50,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F50:O50,F50:O50,"&gt;=0",F50:O50,"&lt;=20")))</f>
+        <f>IF(P50="","",SUMIFS(F50:O50,F50:O50,"&gt;=0",F50:O50,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R50" s="15">
@@ -2979,11 +2948,11 @@
       <c r="N51" s="14" t="n"/>
       <c r="O51" s="14" t="n"/>
       <c r="P51" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F51:O51,'Conversión'!$A$5:$A$8)),COUNTIFS(F51:O51,"&gt;=0",F51:O51,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F51:O51,'Conversión'!$A$5:$A$8)),COUNTIFS(F51:O51,"&gt;=0",F51:O51,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F51:O51,"&gt;=0",F51:O51,"&lt;=20")=0,"",COUNTIFS(F51:O51,"&gt;=0",F51:O51,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q51" s="15">
-        <f>IF(P51="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F51:O51,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F51:O51,F51:O51,"&gt;=0",F51:O51,"&lt;=20")))</f>
+        <f>IF(P51="","",SUMIFS(F51:O51,F51:O51,"&gt;=0",F51:O51,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R51" s="15">
@@ -3016,11 +2985,11 @@
       <c r="N52" s="14" t="n"/>
       <c r="O52" s="14" t="n"/>
       <c r="P52" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F52:O52,'Conversión'!$A$5:$A$8)),COUNTIFS(F52:O52,"&gt;=0",F52:O52,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F52:O52,'Conversión'!$A$5:$A$8)),COUNTIFS(F52:O52,"&gt;=0",F52:O52,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F52:O52,"&gt;=0",F52:O52,"&lt;=20")=0,"",COUNTIFS(F52:O52,"&gt;=0",F52:O52,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q52" s="15">
-        <f>IF(P52="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F52:O52,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F52:O52,F52:O52,"&gt;=0",F52:O52,"&lt;=20")))</f>
+        <f>IF(P52="","",SUMIFS(F52:O52,F52:O52,"&gt;=0",F52:O52,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R52" s="15">
@@ -3053,11 +3022,11 @@
       <c r="N53" s="14" t="n"/>
       <c r="O53" s="14" t="n"/>
       <c r="P53" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F53:O53,'Conversión'!$A$5:$A$8)),COUNTIFS(F53:O53,"&gt;=0",F53:O53,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F53:O53,'Conversión'!$A$5:$A$8)),COUNTIFS(F53:O53,"&gt;=0",F53:O53,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F53:O53,"&gt;=0",F53:O53,"&lt;=20")=0,"",COUNTIFS(F53:O53,"&gt;=0",F53:O53,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q53" s="15">
-        <f>IF(P53="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F53:O53,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F53:O53,F53:O53,"&gt;=0",F53:O53,"&lt;=20")))</f>
+        <f>IF(P53="","",SUMIFS(F53:O53,F53:O53,"&gt;=0",F53:O53,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R53" s="15">
@@ -3090,11 +3059,11 @@
       <c r="N54" s="14" t="n"/>
       <c r="O54" s="14" t="n"/>
       <c r="P54" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F54:O54,'Conversión'!$A$5:$A$8)),COUNTIFS(F54:O54,"&gt;=0",F54:O54,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F54:O54,'Conversión'!$A$5:$A$8)),COUNTIFS(F54:O54,"&gt;=0",F54:O54,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F54:O54,"&gt;=0",F54:O54,"&lt;=20")=0,"",COUNTIFS(F54:O54,"&gt;=0",F54:O54,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q54" s="15">
-        <f>IF(P54="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F54:O54,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F54:O54,F54:O54,"&gt;=0",F54:O54,"&lt;=20")))</f>
+        <f>IF(P54="","",SUMIFS(F54:O54,F54:O54,"&gt;=0",F54:O54,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R54" s="15">
@@ -3127,11 +3096,11 @@
       <c r="N55" s="14" t="n"/>
       <c r="O55" s="14" t="n"/>
       <c r="P55" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F55:O55,'Conversión'!$A$5:$A$8)),COUNTIFS(F55:O55,"&gt;=0",F55:O55,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F55:O55,'Conversión'!$A$5:$A$8)),COUNTIFS(F55:O55,"&gt;=0",F55:O55,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F55:O55,"&gt;=0",F55:O55,"&lt;=20")=0,"",COUNTIFS(F55:O55,"&gt;=0",F55:O55,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q55" s="15">
-        <f>IF(P55="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F55:O55,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F55:O55,F55:O55,"&gt;=0",F55:O55,"&lt;=20")))</f>
+        <f>IF(P55="","",SUMIFS(F55:O55,F55:O55,"&gt;=0",F55:O55,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R55" s="15">
@@ -3164,11 +3133,11 @@
       <c r="N56" s="14" t="n"/>
       <c r="O56" s="14" t="n"/>
       <c r="P56" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F56:O56,'Conversión'!$A$5:$A$8)),COUNTIFS(F56:O56,"&gt;=0",F56:O56,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F56:O56,'Conversión'!$A$5:$A$8)),COUNTIFS(F56:O56,"&gt;=0",F56:O56,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F56:O56,"&gt;=0",F56:O56,"&lt;=20")=0,"",COUNTIFS(F56:O56,"&gt;=0",F56:O56,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q56" s="15">
-        <f>IF(P56="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F56:O56,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F56:O56,F56:O56,"&gt;=0",F56:O56,"&lt;=20")))</f>
+        <f>IF(P56="","",SUMIFS(F56:O56,F56:O56,"&gt;=0",F56:O56,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R56" s="15">
@@ -3201,11 +3170,11 @@
       <c r="N57" s="14" t="n"/>
       <c r="O57" s="14" t="n"/>
       <c r="P57" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F57:O57,'Conversión'!$A$5:$A$8)),COUNTIFS(F57:O57,"&gt;=0",F57:O57,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F57:O57,'Conversión'!$A$5:$A$8)),COUNTIFS(F57:O57,"&gt;=0",F57:O57,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F57:O57,"&gt;=0",F57:O57,"&lt;=20")=0,"",COUNTIFS(F57:O57,"&gt;=0",F57:O57,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q57" s="15">
-        <f>IF(P57="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F57:O57,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F57:O57,F57:O57,"&gt;=0",F57:O57,"&lt;=20")))</f>
+        <f>IF(P57="","",SUMIFS(F57:O57,F57:O57,"&gt;=0",F57:O57,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R57" s="15">
@@ -3238,11 +3207,11 @@
       <c r="N58" s="14" t="n"/>
       <c r="O58" s="14" t="n"/>
       <c r="P58" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F58:O58,'Conversión'!$A$5:$A$8)),COUNTIFS(F58:O58,"&gt;=0",F58:O58,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F58:O58,'Conversión'!$A$5:$A$8)),COUNTIFS(F58:O58,"&gt;=0",F58:O58,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F58:O58,"&gt;=0",F58:O58,"&lt;=20")=0,"",COUNTIFS(F58:O58,"&gt;=0",F58:O58,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q58" s="15">
-        <f>IF(P58="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F58:O58,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F58:O58,F58:O58,"&gt;=0",F58:O58,"&lt;=20")))</f>
+        <f>IF(P58="","",SUMIFS(F58:O58,F58:O58,"&gt;=0",F58:O58,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R58" s="15">
@@ -3275,11 +3244,11 @@
       <c r="N59" s="14" t="n"/>
       <c r="O59" s="14" t="n"/>
       <c r="P59" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F59:O59,'Conversión'!$A$5:$A$8)),COUNTIFS(F59:O59,"&gt;=0",F59:O59,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F59:O59,'Conversión'!$A$5:$A$8)),COUNTIFS(F59:O59,"&gt;=0",F59:O59,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F59:O59,"&gt;=0",F59:O59,"&lt;=20")=0,"",COUNTIFS(F59:O59,"&gt;=0",F59:O59,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q59" s="15">
-        <f>IF(P59="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F59:O59,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F59:O59,F59:O59,"&gt;=0",F59:O59,"&lt;=20")))</f>
+        <f>IF(P59="","",SUMIFS(F59:O59,F59:O59,"&gt;=0",F59:O59,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R59" s="15">
@@ -3312,11 +3281,11 @@
       <c r="N60" s="14" t="n"/>
       <c r="O60" s="14" t="n"/>
       <c r="P60" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F60:O60,'Conversión'!$A$5:$A$8)),COUNTIFS(F60:O60,"&gt;=0",F60:O60,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F60:O60,'Conversión'!$A$5:$A$8)),COUNTIFS(F60:O60,"&gt;=0",F60:O60,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F60:O60,"&gt;=0",F60:O60,"&lt;=20")=0,"",COUNTIFS(F60:O60,"&gt;=0",F60:O60,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q60" s="15">
-        <f>IF(P60="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F60:O60,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F60:O60,F60:O60,"&gt;=0",F60:O60,"&lt;=20")))</f>
+        <f>IF(P60="","",SUMIFS(F60:O60,F60:O60,"&gt;=0",F60:O60,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R60" s="15">
@@ -3349,11 +3318,11 @@
       <c r="N61" s="14" t="n"/>
       <c r="O61" s="14" t="n"/>
       <c r="P61" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F61:O61,'Conversión'!$A$5:$A$8)),COUNTIFS(F61:O61,"&gt;=0",F61:O61,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F61:O61,'Conversión'!$A$5:$A$8)),COUNTIFS(F61:O61,"&gt;=0",F61:O61,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F61:O61,"&gt;=0",F61:O61,"&lt;=20")=0,"",COUNTIFS(F61:O61,"&gt;=0",F61:O61,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q61" s="15">
-        <f>IF(P61="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F61:O61,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F61:O61,F61:O61,"&gt;=0",F61:O61,"&lt;=20")))</f>
+        <f>IF(P61="","",SUMIFS(F61:O61,F61:O61,"&gt;=0",F61:O61,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R61" s="15">
@@ -3386,11 +3355,11 @@
       <c r="N62" s="14" t="n"/>
       <c r="O62" s="14" t="n"/>
       <c r="P62" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F62:O62,'Conversión'!$A$5:$A$8)),COUNTIFS(F62:O62,"&gt;=0",F62:O62,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F62:O62,'Conversión'!$A$5:$A$8)),COUNTIFS(F62:O62,"&gt;=0",F62:O62,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F62:O62,"&gt;=0",F62:O62,"&lt;=20")=0,"",COUNTIFS(F62:O62,"&gt;=0",F62:O62,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q62" s="15">
-        <f>IF(P62="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F62:O62,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F62:O62,F62:O62,"&gt;=0",F62:O62,"&lt;=20")))</f>
+        <f>IF(P62="","",SUMIFS(F62:O62,F62:O62,"&gt;=0",F62:O62,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R62" s="15">
@@ -3423,11 +3392,11 @@
       <c r="N63" s="14" t="n"/>
       <c r="O63" s="14" t="n"/>
       <c r="P63" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F63:O63,'Conversión'!$A$5:$A$8)),COUNTIFS(F63:O63,"&gt;=0",F63:O63,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F63:O63,'Conversión'!$A$5:$A$8)),COUNTIFS(F63:O63,"&gt;=0",F63:O63,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F63:O63,"&gt;=0",F63:O63,"&lt;=20")=0,"",COUNTIFS(F63:O63,"&gt;=0",F63:O63,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q63" s="15">
-        <f>IF(P63="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F63:O63,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F63:O63,F63:O63,"&gt;=0",F63:O63,"&lt;=20")))</f>
+        <f>IF(P63="","",SUMIFS(F63:O63,F63:O63,"&gt;=0",F63:O63,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R63" s="15">
@@ -3460,11 +3429,11 @@
       <c r="N64" s="14" t="n"/>
       <c r="O64" s="14" t="n"/>
       <c r="P64" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F64:O64,'Conversión'!$A$5:$A$8)),COUNTIFS(F64:O64,"&gt;=0",F64:O64,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F64:O64,'Conversión'!$A$5:$A$8)),COUNTIFS(F64:O64,"&gt;=0",F64:O64,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F64:O64,"&gt;=0",F64:O64,"&lt;=20")=0,"",COUNTIFS(F64:O64,"&gt;=0",F64:O64,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q64" s="15">
-        <f>IF(P64="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F64:O64,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F64:O64,F64:O64,"&gt;=0",F64:O64,"&lt;=20")))</f>
+        <f>IF(P64="","",SUMIFS(F64:O64,F64:O64,"&gt;=0",F64:O64,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R64" s="15">
@@ -3497,11 +3466,11 @@
       <c r="N65" s="14" t="n"/>
       <c r="O65" s="14" t="n"/>
       <c r="P65" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F65:O65,'Conversión'!$A$5:$A$8)),COUNTIFS(F65:O65,"&gt;=0",F65:O65,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F65:O65,'Conversión'!$A$5:$A$8)),COUNTIFS(F65:O65,"&gt;=0",F65:O65,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F65:O65,"&gt;=0",F65:O65,"&lt;=20")=0,"",COUNTIFS(F65:O65,"&gt;=0",F65:O65,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q65" s="15">
-        <f>IF(P65="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F65:O65,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F65:O65,F65:O65,"&gt;=0",F65:O65,"&lt;=20")))</f>
+        <f>IF(P65="","",SUMIFS(F65:O65,F65:O65,"&gt;=0",F65:O65,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R65" s="15">
@@ -3534,11 +3503,11 @@
       <c r="N66" s="14" t="n"/>
       <c r="O66" s="14" t="n"/>
       <c r="P66" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F66:O66,'Conversión'!$A$5:$A$8)),COUNTIFS(F66:O66,"&gt;=0",F66:O66,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F66:O66,'Conversión'!$A$5:$A$8)),COUNTIFS(F66:O66,"&gt;=0",F66:O66,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F66:O66,"&gt;=0",F66:O66,"&lt;=20")=0,"",COUNTIFS(F66:O66,"&gt;=0",F66:O66,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q66" s="15">
-        <f>IF(P66="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F66:O66,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F66:O66,F66:O66,"&gt;=0",F66:O66,"&lt;=20")))</f>
+        <f>IF(P66="","",SUMIFS(F66:O66,F66:O66,"&gt;=0",F66:O66,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R66" s="15">
@@ -3571,11 +3540,11 @@
       <c r="N67" s="14" t="n"/>
       <c r="O67" s="14" t="n"/>
       <c r="P67" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F67:O67,'Conversión'!$A$5:$A$8)),COUNTIFS(F67:O67,"&gt;=0",F67:O67,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F67:O67,'Conversión'!$A$5:$A$8)),COUNTIFS(F67:O67,"&gt;=0",F67:O67,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F67:O67,"&gt;=0",F67:O67,"&lt;=20")=0,"",COUNTIFS(F67:O67,"&gt;=0",F67:O67,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q67" s="15">
-        <f>IF(P67="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F67:O67,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F67:O67,F67:O67,"&gt;=0",F67:O67,"&lt;=20")))</f>
+        <f>IF(P67="","",SUMIFS(F67:O67,F67:O67,"&gt;=0",F67:O67,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R67" s="15">
@@ -3608,11 +3577,11 @@
       <c r="N68" s="14" t="n"/>
       <c r="O68" s="14" t="n"/>
       <c r="P68" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F68:O68,'Conversión'!$A$5:$A$8)),COUNTIFS(F68:O68,"&gt;=0",F68:O68,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F68:O68,'Conversión'!$A$5:$A$8)),COUNTIFS(F68:O68,"&gt;=0",F68:O68,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F68:O68,"&gt;=0",F68:O68,"&lt;=20")=0,"",COUNTIFS(F68:O68,"&gt;=0",F68:O68,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q68" s="15">
-        <f>IF(P68="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F68:O68,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F68:O68,F68:O68,"&gt;=0",F68:O68,"&lt;=20")))</f>
+        <f>IF(P68="","",SUMIFS(F68:O68,F68:O68,"&gt;=0",F68:O68,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R68" s="15">
@@ -3645,11 +3614,11 @@
       <c r="N69" s="14" t="n"/>
       <c r="O69" s="14" t="n"/>
       <c r="P69" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F69:O69,'Conversión'!$A$5:$A$8)),COUNTIFS(F69:O69,"&gt;=0",F69:O69,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F69:O69,'Conversión'!$A$5:$A$8)),COUNTIFS(F69:O69,"&gt;=0",F69:O69,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F69:O69,"&gt;=0",F69:O69,"&lt;=20")=0,"",COUNTIFS(F69:O69,"&gt;=0",F69:O69,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q69" s="15">
-        <f>IF(P69="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F69:O69,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F69:O69,F69:O69,"&gt;=0",F69:O69,"&lt;=20")))</f>
+        <f>IF(P69="","",SUMIFS(F69:O69,F69:O69,"&gt;=0",F69:O69,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R69" s="15">
@@ -3682,11 +3651,11 @@
       <c r="N70" s="14" t="n"/>
       <c r="O70" s="14" t="n"/>
       <c r="P70" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F70:O70,'Conversión'!$A$5:$A$8)),COUNTIFS(F70:O70,"&gt;=0",F70:O70,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F70:O70,'Conversión'!$A$5:$A$8)),COUNTIFS(F70:O70,"&gt;=0",F70:O70,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F70:O70,"&gt;=0",F70:O70,"&lt;=20")=0,"",COUNTIFS(F70:O70,"&gt;=0",F70:O70,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q70" s="15">
-        <f>IF(P70="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F70:O70,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F70:O70,F70:O70,"&gt;=0",F70:O70,"&lt;=20")))</f>
+        <f>IF(P70="","",SUMIFS(F70:O70,F70:O70,"&gt;=0",F70:O70,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R70" s="15">
@@ -3719,11 +3688,11 @@
       <c r="N71" s="14" t="n"/>
       <c r="O71" s="14" t="n"/>
       <c r="P71" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F71:O71,'Conversión'!$A$5:$A$8)),COUNTIFS(F71:O71,"&gt;=0",F71:O71,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F71:O71,'Conversión'!$A$5:$A$8)),COUNTIFS(F71:O71,"&gt;=0",F71:O71,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F71:O71,"&gt;=0",F71:O71,"&lt;=20")=0,"",COUNTIFS(F71:O71,"&gt;=0",F71:O71,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q71" s="15">
-        <f>IF(P71="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F71:O71,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F71:O71,F71:O71,"&gt;=0",F71:O71,"&lt;=20")))</f>
+        <f>IF(P71="","",SUMIFS(F71:O71,F71:O71,"&gt;=0",F71:O71,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R71" s="15">
@@ -3756,11 +3725,11 @@
       <c r="N72" s="14" t="n"/>
       <c r="O72" s="14" t="n"/>
       <c r="P72" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F72:O72,'Conversión'!$A$5:$A$8)),COUNTIFS(F72:O72,"&gt;=0",F72:O72,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F72:O72,'Conversión'!$A$5:$A$8)),COUNTIFS(F72:O72,"&gt;=0",F72:O72,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F72:O72,"&gt;=0",F72:O72,"&lt;=20")=0,"",COUNTIFS(F72:O72,"&gt;=0",F72:O72,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q72" s="15">
-        <f>IF(P72="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F72:O72,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F72:O72,F72:O72,"&gt;=0",F72:O72,"&lt;=20")))</f>
+        <f>IF(P72="","",SUMIFS(F72:O72,F72:O72,"&gt;=0",F72:O72,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R72" s="15">
@@ -3793,11 +3762,11 @@
       <c r="N73" s="14" t="n"/>
       <c r="O73" s="14" t="n"/>
       <c r="P73" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F73:O73,'Conversión'!$A$5:$A$8)),COUNTIFS(F73:O73,"&gt;=0",F73:O73,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F73:O73,'Conversión'!$A$5:$A$8)),COUNTIFS(F73:O73,"&gt;=0",F73:O73,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F73:O73,"&gt;=0",F73:O73,"&lt;=20")=0,"",COUNTIFS(F73:O73,"&gt;=0",F73:O73,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q73" s="15">
-        <f>IF(P73="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F73:O73,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F73:O73,F73:O73,"&gt;=0",F73:O73,"&lt;=20")))</f>
+        <f>IF(P73="","",SUMIFS(F73:O73,F73:O73,"&gt;=0",F73:O73,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R73" s="15">
@@ -3830,11 +3799,11 @@
       <c r="N74" s="14" t="n"/>
       <c r="O74" s="14" t="n"/>
       <c r="P74" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F74:O74,'Conversión'!$A$5:$A$8)),COUNTIFS(F74:O74,"&gt;=0",F74:O74,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F74:O74,'Conversión'!$A$5:$A$8)),COUNTIFS(F74:O74,"&gt;=0",F74:O74,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F74:O74,"&gt;=0",F74:O74,"&lt;=20")=0,"",COUNTIFS(F74:O74,"&gt;=0",F74:O74,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q74" s="15">
-        <f>IF(P74="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F74:O74,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F74:O74,F74:O74,"&gt;=0",F74:O74,"&lt;=20")))</f>
+        <f>IF(P74="","",SUMIFS(F74:O74,F74:O74,"&gt;=0",F74:O74,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R74" s="15">
@@ -3867,11 +3836,11 @@
       <c r="N75" s="14" t="n"/>
       <c r="O75" s="14" t="n"/>
       <c r="P75" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F75:O75,'Conversión'!$A$5:$A$8)),COUNTIFS(F75:O75,"&gt;=0",F75:O75,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F75:O75,'Conversión'!$A$5:$A$8)),COUNTIFS(F75:O75,"&gt;=0",F75:O75,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F75:O75,"&gt;=0",F75:O75,"&lt;=20")=0,"",COUNTIFS(F75:O75,"&gt;=0",F75:O75,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q75" s="15">
-        <f>IF(P75="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F75:O75,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F75:O75,F75:O75,"&gt;=0",F75:O75,"&lt;=20")))</f>
+        <f>IF(P75="","",SUMIFS(F75:O75,F75:O75,"&gt;=0",F75:O75,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R75" s="15">
@@ -3904,11 +3873,11 @@
       <c r="N76" s="14" t="n"/>
       <c r="O76" s="14" t="n"/>
       <c r="P76" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F76:O76,'Conversión'!$A$5:$A$8)),COUNTIFS(F76:O76,"&gt;=0",F76:O76,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F76:O76,'Conversión'!$A$5:$A$8)),COUNTIFS(F76:O76,"&gt;=0",F76:O76,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F76:O76,"&gt;=0",F76:O76,"&lt;=20")=0,"",COUNTIFS(F76:O76,"&gt;=0",F76:O76,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q76" s="15">
-        <f>IF(P76="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F76:O76,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F76:O76,F76:O76,"&gt;=0",F76:O76,"&lt;=20")))</f>
+        <f>IF(P76="","",SUMIFS(F76:O76,F76:O76,"&gt;=0",F76:O76,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R76" s="15">
@@ -3941,11 +3910,11 @@
       <c r="N77" s="14" t="n"/>
       <c r="O77" s="14" t="n"/>
       <c r="P77" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F77:O77,'Conversión'!$A$5:$A$8)),COUNTIFS(F77:O77,"&gt;=0",F77:O77,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F77:O77,'Conversión'!$A$5:$A$8)),COUNTIFS(F77:O77,"&gt;=0",F77:O77,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F77:O77,"&gt;=0",F77:O77,"&lt;=20")=0,"",COUNTIFS(F77:O77,"&gt;=0",F77:O77,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q77" s="15">
-        <f>IF(P77="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F77:O77,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F77:O77,F77:O77,"&gt;=0",F77:O77,"&lt;=20")))</f>
+        <f>IF(P77="","",SUMIFS(F77:O77,F77:O77,"&gt;=0",F77:O77,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R77" s="15">
@@ -3978,11 +3947,11 @@
       <c r="N78" s="14" t="n"/>
       <c r="O78" s="14" t="n"/>
       <c r="P78" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F78:O78,'Conversión'!$A$5:$A$8)),COUNTIFS(F78:O78,"&gt;=0",F78:O78,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F78:O78,'Conversión'!$A$5:$A$8)),COUNTIFS(F78:O78,"&gt;=0",F78:O78,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F78:O78,"&gt;=0",F78:O78,"&lt;=20")=0,"",COUNTIFS(F78:O78,"&gt;=0",F78:O78,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q78" s="15">
-        <f>IF(P78="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F78:O78,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F78:O78,F78:O78,"&gt;=0",F78:O78,"&lt;=20")))</f>
+        <f>IF(P78="","",SUMIFS(F78:O78,F78:O78,"&gt;=0",F78:O78,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R78" s="15">
@@ -4015,11 +3984,11 @@
       <c r="N79" s="14" t="n"/>
       <c r="O79" s="14" t="n"/>
       <c r="P79" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F79:O79,'Conversión'!$A$5:$A$8)),COUNTIFS(F79:O79,"&gt;=0",F79:O79,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F79:O79,'Conversión'!$A$5:$A$8)),COUNTIFS(F79:O79,"&gt;=0",F79:O79,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F79:O79,"&gt;=0",F79:O79,"&lt;=20")=0,"",COUNTIFS(F79:O79,"&gt;=0",F79:O79,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q79" s="15">
-        <f>IF(P79="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F79:O79,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F79:O79,F79:O79,"&gt;=0",F79:O79,"&lt;=20")))</f>
+        <f>IF(P79="","",SUMIFS(F79:O79,F79:O79,"&gt;=0",F79:O79,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R79" s="15">
@@ -4052,11 +4021,11 @@
       <c r="N80" s="14" t="n"/>
       <c r="O80" s="14" t="n"/>
       <c r="P80" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F80:O80,'Conversión'!$A$5:$A$8)),COUNTIFS(F80:O80,"&gt;=0",F80:O80,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F80:O80,'Conversión'!$A$5:$A$8)),COUNTIFS(F80:O80,"&gt;=0",F80:O80,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F80:O80,"&gt;=0",F80:O80,"&lt;=20")=0,"",COUNTIFS(F80:O80,"&gt;=0",F80:O80,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q80" s="15">
-        <f>IF(P80="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F80:O80,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F80:O80,F80:O80,"&gt;=0",F80:O80,"&lt;=20")))</f>
+        <f>IF(P80="","",SUMIFS(F80:O80,F80:O80,"&gt;=0",F80:O80,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R80" s="15">
@@ -4089,11 +4058,11 @@
       <c r="N81" s="14" t="n"/>
       <c r="O81" s="14" t="n"/>
       <c r="P81" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F81:O81,'Conversión'!$A$5:$A$8)),COUNTIFS(F81:O81,"&gt;=0",F81:O81,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F81:O81,'Conversión'!$A$5:$A$8)),COUNTIFS(F81:O81,"&gt;=0",F81:O81,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F81:O81,"&gt;=0",F81:O81,"&lt;=20")=0,"",COUNTIFS(F81:O81,"&gt;=0",F81:O81,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q81" s="15">
-        <f>IF(P81="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F81:O81,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F81:O81,F81:O81,"&gt;=0",F81:O81,"&lt;=20")))</f>
+        <f>IF(P81="","",SUMIFS(F81:O81,F81:O81,"&gt;=0",F81:O81,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R81" s="15">
@@ -4126,11 +4095,11 @@
       <c r="N82" s="14" t="n"/>
       <c r="O82" s="14" t="n"/>
       <c r="P82" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F82:O82,'Conversión'!$A$5:$A$8)),COUNTIFS(F82:O82,"&gt;=0",F82:O82,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F82:O82,'Conversión'!$A$5:$A$8)),COUNTIFS(F82:O82,"&gt;=0",F82:O82,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F82:O82,"&gt;=0",F82:O82,"&lt;=20")=0,"",COUNTIFS(F82:O82,"&gt;=0",F82:O82,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q82" s="15">
-        <f>IF(P82="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F82:O82,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F82:O82,F82:O82,"&gt;=0",F82:O82,"&lt;=20")))</f>
+        <f>IF(P82="","",SUMIFS(F82:O82,F82:O82,"&gt;=0",F82:O82,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R82" s="15">
@@ -4163,11 +4132,11 @@
       <c r="N83" s="14" t="n"/>
       <c r="O83" s="14" t="n"/>
       <c r="P83" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F83:O83,'Conversión'!$A$5:$A$8)),COUNTIFS(F83:O83,"&gt;=0",F83:O83,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F83:O83,'Conversión'!$A$5:$A$8)),COUNTIFS(F83:O83,"&gt;=0",F83:O83,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F83:O83,"&gt;=0",F83:O83,"&lt;=20")=0,"",COUNTIFS(F83:O83,"&gt;=0",F83:O83,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q83" s="15">
-        <f>IF(P83="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F83:O83,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F83:O83,F83:O83,"&gt;=0",F83:O83,"&lt;=20")))</f>
+        <f>IF(P83="","",SUMIFS(F83:O83,F83:O83,"&gt;=0",F83:O83,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R83" s="15">
@@ -4200,11 +4169,11 @@
       <c r="N84" s="14" t="n"/>
       <c r="O84" s="14" t="n"/>
       <c r="P84" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F84:O84,'Conversión'!$A$5:$A$8)),COUNTIFS(F84:O84,"&gt;=0",F84:O84,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F84:O84,'Conversión'!$A$5:$A$8)),COUNTIFS(F84:O84,"&gt;=0",F84:O84,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F84:O84,"&gt;=0",F84:O84,"&lt;=20")=0,"",COUNTIFS(F84:O84,"&gt;=0",F84:O84,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q84" s="15">
-        <f>IF(P84="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F84:O84,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F84:O84,F84:O84,"&gt;=0",F84:O84,"&lt;=20")))</f>
+        <f>IF(P84="","",SUMIFS(F84:O84,F84:O84,"&gt;=0",F84:O84,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R84" s="15">
@@ -4237,11 +4206,11 @@
       <c r="N85" s="14" t="n"/>
       <c r="O85" s="14" t="n"/>
       <c r="P85" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F85:O85,'Conversión'!$A$5:$A$8)),COUNTIFS(F85:O85,"&gt;=0",F85:O85,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F85:O85,'Conversión'!$A$5:$A$8)),COUNTIFS(F85:O85,"&gt;=0",F85:O85,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F85:O85,"&gt;=0",F85:O85,"&lt;=20")=0,"",COUNTIFS(F85:O85,"&gt;=0",F85:O85,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q85" s="15">
-        <f>IF(P85="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F85:O85,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F85:O85,F85:O85,"&gt;=0",F85:O85,"&lt;=20")))</f>
+        <f>IF(P85="","",SUMIFS(F85:O85,F85:O85,"&gt;=0",F85:O85,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R85" s="15">
@@ -4274,11 +4243,11 @@
       <c r="N86" s="14" t="n"/>
       <c r="O86" s="14" t="n"/>
       <c r="P86" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F86:O86,'Conversión'!$A$5:$A$8)),COUNTIFS(F86:O86,"&gt;=0",F86:O86,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F86:O86,'Conversión'!$A$5:$A$8)),COUNTIFS(F86:O86,"&gt;=0",F86:O86,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F86:O86,"&gt;=0",F86:O86,"&lt;=20")=0,"",COUNTIFS(F86:O86,"&gt;=0",F86:O86,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q86" s="15">
-        <f>IF(P86="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F86:O86,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F86:O86,F86:O86,"&gt;=0",F86:O86,"&lt;=20")))</f>
+        <f>IF(P86="","",SUMIFS(F86:O86,F86:O86,"&gt;=0",F86:O86,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R86" s="15">
@@ -4311,11 +4280,11 @@
       <c r="N87" s="14" t="n"/>
       <c r="O87" s="14" t="n"/>
       <c r="P87" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F87:O87,'Conversión'!$A$5:$A$8)),COUNTIFS(F87:O87,"&gt;=0",F87:O87,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F87:O87,'Conversión'!$A$5:$A$8)),COUNTIFS(F87:O87,"&gt;=0",F87:O87,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F87:O87,"&gt;=0",F87:O87,"&lt;=20")=0,"",COUNTIFS(F87:O87,"&gt;=0",F87:O87,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q87" s="15">
-        <f>IF(P87="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F87:O87,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F87:O87,F87:O87,"&gt;=0",F87:O87,"&lt;=20")))</f>
+        <f>IF(P87="","",SUMIFS(F87:O87,F87:O87,"&gt;=0",F87:O87,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R87" s="15">
@@ -4348,11 +4317,11 @@
       <c r="N88" s="14" t="n"/>
       <c r="O88" s="14" t="n"/>
       <c r="P88" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F88:O88,'Conversión'!$A$5:$A$8)),COUNTIFS(F88:O88,"&gt;=0",F88:O88,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F88:O88,'Conversión'!$A$5:$A$8)),COUNTIFS(F88:O88,"&gt;=0",F88:O88,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F88:O88,"&gt;=0",F88:O88,"&lt;=20")=0,"",COUNTIFS(F88:O88,"&gt;=0",F88:O88,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q88" s="15">
-        <f>IF(P88="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F88:O88,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F88:O88,F88:O88,"&gt;=0",F88:O88,"&lt;=20")))</f>
+        <f>IF(P88="","",SUMIFS(F88:O88,F88:O88,"&gt;=0",F88:O88,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R88" s="15">
@@ -4385,11 +4354,11 @@
       <c r="N89" s="14" t="n"/>
       <c r="O89" s="14" t="n"/>
       <c r="P89" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F89:O89,'Conversión'!$A$5:$A$8)),COUNTIFS(F89:O89,"&gt;=0",F89:O89,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F89:O89,'Conversión'!$A$5:$A$8)),COUNTIFS(F89:O89,"&gt;=0",F89:O89,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F89:O89,"&gt;=0",F89:O89,"&lt;=20")=0,"",COUNTIFS(F89:O89,"&gt;=0",F89:O89,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q89" s="15">
-        <f>IF(P89="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F89:O89,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F89:O89,F89:O89,"&gt;=0",F89:O89,"&lt;=20")))</f>
+        <f>IF(P89="","",SUMIFS(F89:O89,F89:O89,"&gt;=0",F89:O89,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R89" s="15">
@@ -4422,11 +4391,11 @@
       <c r="N90" s="14" t="n"/>
       <c r="O90" s="14" t="n"/>
       <c r="P90" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F90:O90,'Conversión'!$A$5:$A$8)),COUNTIFS(F90:O90,"&gt;=0",F90:O90,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F90:O90,'Conversión'!$A$5:$A$8)),COUNTIFS(F90:O90,"&gt;=0",F90:O90,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F90:O90,"&gt;=0",F90:O90,"&lt;=20")=0,"",COUNTIFS(F90:O90,"&gt;=0",F90:O90,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q90" s="15">
-        <f>IF(P90="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F90:O90,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F90:O90,F90:O90,"&gt;=0",F90:O90,"&lt;=20")))</f>
+        <f>IF(P90="","",SUMIFS(F90:O90,F90:O90,"&gt;=0",F90:O90,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R90" s="15">
@@ -4459,11 +4428,11 @@
       <c r="N91" s="14" t="n"/>
       <c r="O91" s="14" t="n"/>
       <c r="P91" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F91:O91,'Conversión'!$A$5:$A$8)),COUNTIFS(F91:O91,"&gt;=0",F91:O91,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F91:O91,'Conversión'!$A$5:$A$8)),COUNTIFS(F91:O91,"&gt;=0",F91:O91,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F91:O91,"&gt;=0",F91:O91,"&lt;=20")=0,"",COUNTIFS(F91:O91,"&gt;=0",F91:O91,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q91" s="15">
-        <f>IF(P91="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F91:O91,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F91:O91,F91:O91,"&gt;=0",F91:O91,"&lt;=20")))</f>
+        <f>IF(P91="","",SUMIFS(F91:O91,F91:O91,"&gt;=0",F91:O91,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R91" s="15">
@@ -4496,11 +4465,11 @@
       <c r="N92" s="14" t="n"/>
       <c r="O92" s="14" t="n"/>
       <c r="P92" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F92:O92,'Conversión'!$A$5:$A$8)),COUNTIFS(F92:O92,"&gt;=0",F92:O92,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F92:O92,'Conversión'!$A$5:$A$8)),COUNTIFS(F92:O92,"&gt;=0",F92:O92,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F92:O92,"&gt;=0",F92:O92,"&lt;=20")=0,"",COUNTIFS(F92:O92,"&gt;=0",F92:O92,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q92" s="15">
-        <f>IF(P92="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F92:O92,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F92:O92,F92:O92,"&gt;=0",F92:O92,"&lt;=20")))</f>
+        <f>IF(P92="","",SUMIFS(F92:O92,F92:O92,"&gt;=0",F92:O92,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R92" s="15">
@@ -4533,11 +4502,11 @@
       <c r="N93" s="14" t="n"/>
       <c r="O93" s="14" t="n"/>
       <c r="P93" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F93:O93,'Conversión'!$A$5:$A$8)),COUNTIFS(F93:O93,"&gt;=0",F93:O93,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F93:O93,'Conversión'!$A$5:$A$8)),COUNTIFS(F93:O93,"&gt;=0",F93:O93,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F93:O93,"&gt;=0",F93:O93,"&lt;=20")=0,"",COUNTIFS(F93:O93,"&gt;=0",F93:O93,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q93" s="15">
-        <f>IF(P93="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F93:O93,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F93:O93,F93:O93,"&gt;=0",F93:O93,"&lt;=20")))</f>
+        <f>IF(P93="","",SUMIFS(F93:O93,F93:O93,"&gt;=0",F93:O93,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R93" s="15">
@@ -4570,11 +4539,11 @@
       <c r="N94" s="14" t="n"/>
       <c r="O94" s="14" t="n"/>
       <c r="P94" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F94:O94,'Conversión'!$A$5:$A$8)),COUNTIFS(F94:O94,"&gt;=0",F94:O94,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F94:O94,'Conversión'!$A$5:$A$8)),COUNTIFS(F94:O94,"&gt;=0",F94:O94,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F94:O94,"&gt;=0",F94:O94,"&lt;=20")=0,"",COUNTIFS(F94:O94,"&gt;=0",F94:O94,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q94" s="15">
-        <f>IF(P94="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F94:O94,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F94:O94,F94:O94,"&gt;=0",F94:O94,"&lt;=20")))</f>
+        <f>IF(P94="","",SUMIFS(F94:O94,F94:O94,"&gt;=0",F94:O94,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R94" s="15">
@@ -4607,11 +4576,11 @@
       <c r="N95" s="14" t="n"/>
       <c r="O95" s="14" t="n"/>
       <c r="P95" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F95:O95,'Conversión'!$A$5:$A$8)),COUNTIFS(F95:O95,"&gt;=0",F95:O95,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F95:O95,'Conversión'!$A$5:$A$8)),COUNTIFS(F95:O95,"&gt;=0",F95:O95,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F95:O95,"&gt;=0",F95:O95,"&lt;=20")=0,"",COUNTIFS(F95:O95,"&gt;=0",F95:O95,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q95" s="15">
-        <f>IF(P95="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F95:O95,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F95:O95,F95:O95,"&gt;=0",F95:O95,"&lt;=20")))</f>
+        <f>IF(P95="","",SUMIFS(F95:O95,F95:O95,"&gt;=0",F95:O95,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R95" s="15">
@@ -4644,11 +4613,11 @@
       <c r="N96" s="14" t="n"/>
       <c r="O96" s="14" t="n"/>
       <c r="P96" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F96:O96,'Conversión'!$A$5:$A$8)),COUNTIFS(F96:O96,"&gt;=0",F96:O96,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F96:O96,'Conversión'!$A$5:$A$8)),COUNTIFS(F96:O96,"&gt;=0",F96:O96,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F96:O96,"&gt;=0",F96:O96,"&lt;=20")=0,"",COUNTIFS(F96:O96,"&gt;=0",F96:O96,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q96" s="15">
-        <f>IF(P96="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F96:O96,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F96:O96,F96:O96,"&gt;=0",F96:O96,"&lt;=20")))</f>
+        <f>IF(P96="","",SUMIFS(F96:O96,F96:O96,"&gt;=0",F96:O96,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R96" s="15">
@@ -4681,11 +4650,11 @@
       <c r="N97" s="14" t="n"/>
       <c r="O97" s="14" t="n"/>
       <c r="P97" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F97:O97,'Conversión'!$A$5:$A$8)),COUNTIFS(F97:O97,"&gt;=0",F97:O97,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F97:O97,'Conversión'!$A$5:$A$8)),COUNTIFS(F97:O97,"&gt;=0",F97:O97,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F97:O97,"&gt;=0",F97:O97,"&lt;=20")=0,"",COUNTIFS(F97:O97,"&gt;=0",F97:O97,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q97" s="15">
-        <f>IF(P97="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F97:O97,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F97:O97,F97:O97,"&gt;=0",F97:O97,"&lt;=20")))</f>
+        <f>IF(P97="","",SUMIFS(F97:O97,F97:O97,"&gt;=0",F97:O97,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R97" s="15">
@@ -4718,11 +4687,11 @@
       <c r="N98" s="14" t="n"/>
       <c r="O98" s="14" t="n"/>
       <c r="P98" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F98:O98,'Conversión'!$A$5:$A$8)),COUNTIFS(F98:O98,"&gt;=0",F98:O98,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F98:O98,'Conversión'!$A$5:$A$8)),COUNTIFS(F98:O98,"&gt;=0",F98:O98,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F98:O98,"&gt;=0",F98:O98,"&lt;=20")=0,"",COUNTIFS(F98:O98,"&gt;=0",F98:O98,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q98" s="15">
-        <f>IF(P98="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F98:O98,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F98:O98,F98:O98,"&gt;=0",F98:O98,"&lt;=20")))</f>
+        <f>IF(P98="","",SUMIFS(F98:O98,F98:O98,"&gt;=0",F98:O98,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R98" s="15">
@@ -4755,11 +4724,11 @@
       <c r="N99" s="14" t="n"/>
       <c r="O99" s="14" t="n"/>
       <c r="P99" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F99:O99,'Conversión'!$A$5:$A$8)),COUNTIFS(F99:O99,"&gt;=0",F99:O99,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F99:O99,'Conversión'!$A$5:$A$8)),COUNTIFS(F99:O99,"&gt;=0",F99:O99,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F99:O99,"&gt;=0",F99:O99,"&lt;=20")=0,"",COUNTIFS(F99:O99,"&gt;=0",F99:O99,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q99" s="15">
-        <f>IF(P99="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F99:O99,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F99:O99,F99:O99,"&gt;=0",F99:O99,"&lt;=20")))</f>
+        <f>IF(P99="","",SUMIFS(F99:O99,F99:O99,"&gt;=0",F99:O99,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R99" s="15">
@@ -4792,11 +4761,11 @@
       <c r="N100" s="14" t="n"/>
       <c r="O100" s="14" t="n"/>
       <c r="P100" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F100:O100,'Conversión'!$A$5:$A$8)),COUNTIFS(F100:O100,"&gt;=0",F100:O100,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F100:O100,'Conversión'!$A$5:$A$8)),COUNTIFS(F100:O100,"&gt;=0",F100:O100,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F100:O100,"&gt;=0",F100:O100,"&lt;=20")=0,"",COUNTIFS(F100:O100,"&gt;=0",F100:O100,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q100" s="15">
-        <f>IF(P100="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F100:O100,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F100:O100,F100:O100,"&gt;=0",F100:O100,"&lt;=20")))</f>
+        <f>IF(P100="","",SUMIFS(F100:O100,F100:O100,"&gt;=0",F100:O100,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R100" s="15">
@@ -4829,11 +4798,11 @@
       <c r="N101" s="14" t="n"/>
       <c r="O101" s="14" t="n"/>
       <c r="P101" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F101:O101,'Conversión'!$A$5:$A$8)),COUNTIFS(F101:O101,"&gt;=0",F101:O101,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F101:O101,'Conversión'!$A$5:$A$8)),COUNTIFS(F101:O101,"&gt;=0",F101:O101,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F101:O101,"&gt;=0",F101:O101,"&lt;=20")=0,"",COUNTIFS(F101:O101,"&gt;=0",F101:O101,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q101" s="15">
-        <f>IF(P101="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F101:O101,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F101:O101,F101:O101,"&gt;=0",F101:O101,"&lt;=20")))</f>
+        <f>IF(P101="","",SUMIFS(F101:O101,F101:O101,"&gt;=0",F101:O101,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R101" s="15">
@@ -4866,11 +4835,11 @@
       <c r="N102" s="14" t="n"/>
       <c r="O102" s="14" t="n"/>
       <c r="P102" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F102:O102,'Conversión'!$A$5:$A$8)),COUNTIFS(F102:O102,"&gt;=0",F102:O102,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F102:O102,'Conversión'!$A$5:$A$8)),COUNTIFS(F102:O102,"&gt;=0",F102:O102,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F102:O102,"&gt;=0",F102:O102,"&lt;=20")=0,"",COUNTIFS(F102:O102,"&gt;=0",F102:O102,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q102" s="15">
-        <f>IF(P102="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F102:O102,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F102:O102,F102:O102,"&gt;=0",F102:O102,"&lt;=20")))</f>
+        <f>IF(P102="","",SUMIFS(F102:O102,F102:O102,"&gt;=0",F102:O102,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R102" s="15">
@@ -4903,11 +4872,11 @@
       <c r="N103" s="14" t="n"/>
       <c r="O103" s="14" t="n"/>
       <c r="P103" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F103:O103,'Conversión'!$A$5:$A$8)),COUNTIFS(F103:O103,"&gt;=0",F103:O103,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F103:O103,'Conversión'!$A$5:$A$8)),COUNTIFS(F103:O103,"&gt;=0",F103:O103,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F103:O103,"&gt;=0",F103:O103,"&lt;=20")=0,"",COUNTIFS(F103:O103,"&gt;=0",F103:O103,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q103" s="15">
-        <f>IF(P103="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F103:O103,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F103:O103,F103:O103,"&gt;=0",F103:O103,"&lt;=20")))</f>
+        <f>IF(P103="","",SUMIFS(F103:O103,F103:O103,"&gt;=0",F103:O103,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R103" s="15">
@@ -4940,11 +4909,11 @@
       <c r="N104" s="14" t="n"/>
       <c r="O104" s="14" t="n"/>
       <c r="P104" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F104:O104,'Conversión'!$A$5:$A$8)),COUNTIFS(F104:O104,"&gt;=0",F104:O104,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F104:O104,'Conversión'!$A$5:$A$8)),COUNTIFS(F104:O104,"&gt;=0",F104:O104,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F104:O104,"&gt;=0",F104:O104,"&lt;=20")=0,"",COUNTIFS(F104:O104,"&gt;=0",F104:O104,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q104" s="15">
-        <f>IF(P104="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F104:O104,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F104:O104,F104:O104,"&gt;=0",F104:O104,"&lt;=20")))</f>
+        <f>IF(P104="","",SUMIFS(F104:O104,F104:O104,"&gt;=0",F104:O104,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R104" s="15">
@@ -4977,11 +4946,11 @@
       <c r="N105" s="14" t="n"/>
       <c r="O105" s="14" t="n"/>
       <c r="P105" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F105:O105,'Conversión'!$A$5:$A$8)),COUNTIFS(F105:O105,"&gt;=0",F105:O105,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F105:O105,'Conversión'!$A$5:$A$8)),COUNTIFS(F105:O105,"&gt;=0",F105:O105,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F105:O105,"&gt;=0",F105:O105,"&lt;=20")=0,"",COUNTIFS(F105:O105,"&gt;=0",F105:O105,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q105" s="15">
-        <f>IF(P105="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F105:O105,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F105:O105,F105:O105,"&gt;=0",F105:O105,"&lt;=20")))</f>
+        <f>IF(P105="","",SUMIFS(F105:O105,F105:O105,"&gt;=0",F105:O105,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R105" s="15">
@@ -5014,11 +4983,11 @@
       <c r="N106" s="14" t="n"/>
       <c r="O106" s="14" t="n"/>
       <c r="P106" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F106:O106,'Conversión'!$A$5:$A$8)),COUNTIFS(F106:O106,"&gt;=0",F106:O106,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F106:O106,'Conversión'!$A$5:$A$8)),COUNTIFS(F106:O106,"&gt;=0",F106:O106,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F106:O106,"&gt;=0",F106:O106,"&lt;=20")=0,"",COUNTIFS(F106:O106,"&gt;=0",F106:O106,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q106" s="15">
-        <f>IF(P106="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F106:O106,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F106:O106,F106:O106,"&gt;=0",F106:O106,"&lt;=20")))</f>
+        <f>IF(P106="","",SUMIFS(F106:O106,F106:O106,"&gt;=0",F106:O106,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R106" s="15">
@@ -5051,11 +5020,11 @@
       <c r="N107" s="14" t="n"/>
       <c r="O107" s="14" t="n"/>
       <c r="P107" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F107:O107,'Conversión'!$A$5:$A$8)),COUNTIFS(F107:O107,"&gt;=0",F107:O107,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F107:O107,'Conversión'!$A$5:$A$8)),COUNTIFS(F107:O107,"&gt;=0",F107:O107,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F107:O107,"&gt;=0",F107:O107,"&lt;=20")=0,"",COUNTIFS(F107:O107,"&gt;=0",F107:O107,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q107" s="15">
-        <f>IF(P107="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F107:O107,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F107:O107,F107:O107,"&gt;=0",F107:O107,"&lt;=20")))</f>
+        <f>IF(P107="","",SUMIFS(F107:O107,F107:O107,"&gt;=0",F107:O107,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R107" s="15">
@@ -5088,11 +5057,11 @@
       <c r="N108" s="14" t="n"/>
       <c r="O108" s="14" t="n"/>
       <c r="P108" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F108:O108,'Conversión'!$A$5:$A$8)),COUNTIFS(F108:O108,"&gt;=0",F108:O108,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F108:O108,'Conversión'!$A$5:$A$8)),COUNTIFS(F108:O108,"&gt;=0",F108:O108,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F108:O108,"&gt;=0",F108:O108,"&lt;=20")=0,"",COUNTIFS(F108:O108,"&gt;=0",F108:O108,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q108" s="15">
-        <f>IF(P108="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F108:O108,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F108:O108,F108:O108,"&gt;=0",F108:O108,"&lt;=20")))</f>
+        <f>IF(P108="","",SUMIFS(F108:O108,F108:O108,"&gt;=0",F108:O108,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R108" s="15">
@@ -5125,11 +5094,11 @@
       <c r="N109" s="14" t="n"/>
       <c r="O109" s="14" t="n"/>
       <c r="P109" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F109:O109,'Conversión'!$A$5:$A$8)),COUNTIFS(F109:O109,"&gt;=0",F109:O109,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F109:O109,'Conversión'!$A$5:$A$8)),COUNTIFS(F109:O109,"&gt;=0",F109:O109,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F109:O109,"&gt;=0",F109:O109,"&lt;=20")=0,"",COUNTIFS(F109:O109,"&gt;=0",F109:O109,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q109" s="15">
-        <f>IF(P109="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F109:O109,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F109:O109,F109:O109,"&gt;=0",F109:O109,"&lt;=20")))</f>
+        <f>IF(P109="","",SUMIFS(F109:O109,F109:O109,"&gt;=0",F109:O109,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R109" s="15">
@@ -5162,11 +5131,11 @@
       <c r="N110" s="14" t="n"/>
       <c r="O110" s="14" t="n"/>
       <c r="P110" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F110:O110,'Conversión'!$A$5:$A$8)),COUNTIFS(F110:O110,"&gt;=0",F110:O110,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F110:O110,'Conversión'!$A$5:$A$8)),COUNTIFS(F110:O110,"&gt;=0",F110:O110,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F110:O110,"&gt;=0",F110:O110,"&lt;=20")=0,"",COUNTIFS(F110:O110,"&gt;=0",F110:O110,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q110" s="15">
-        <f>IF(P110="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F110:O110,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F110:O110,F110:O110,"&gt;=0",F110:O110,"&lt;=20")))</f>
+        <f>IF(P110="","",SUMIFS(F110:O110,F110:O110,"&gt;=0",F110:O110,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R110" s="15">
@@ -5199,11 +5168,11 @@
       <c r="N111" s="14" t="n"/>
       <c r="O111" s="14" t="n"/>
       <c r="P111" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F111:O111,'Conversión'!$A$5:$A$8)),COUNTIFS(F111:O111,"&gt;=0",F111:O111,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F111:O111,'Conversión'!$A$5:$A$8)),COUNTIFS(F111:O111,"&gt;=0",F111:O111,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F111:O111,"&gt;=0",F111:O111,"&lt;=20")=0,"",COUNTIFS(F111:O111,"&gt;=0",F111:O111,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q111" s="15">
-        <f>IF(P111="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F111:O111,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F111:O111,F111:O111,"&gt;=0",F111:O111,"&lt;=20")))</f>
+        <f>IF(P111="","",SUMIFS(F111:O111,F111:O111,"&gt;=0",F111:O111,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R111" s="15">
@@ -5236,11 +5205,11 @@
       <c r="N112" s="14" t="n"/>
       <c r="O112" s="14" t="n"/>
       <c r="P112" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F112:O112,'Conversión'!$A$5:$A$8)),COUNTIFS(F112:O112,"&gt;=0",F112:O112,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F112:O112,'Conversión'!$A$5:$A$8)),COUNTIFS(F112:O112,"&gt;=0",F112:O112,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F112:O112,"&gt;=0",F112:O112,"&lt;=20")=0,"",COUNTIFS(F112:O112,"&gt;=0",F112:O112,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q112" s="15">
-        <f>IF(P112="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F112:O112,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F112:O112,F112:O112,"&gt;=0",F112:O112,"&lt;=20")))</f>
+        <f>IF(P112="","",SUMIFS(F112:O112,F112:O112,"&gt;=0",F112:O112,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R112" s="15">
@@ -5273,11 +5242,11 @@
       <c r="N113" s="14" t="n"/>
       <c r="O113" s="14" t="n"/>
       <c r="P113" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F113:O113,'Conversión'!$A$5:$A$8)),COUNTIFS(F113:O113,"&gt;=0",F113:O113,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F113:O113,'Conversión'!$A$5:$A$8)),COUNTIFS(F113:O113,"&gt;=0",F113:O113,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F113:O113,"&gt;=0",F113:O113,"&lt;=20")=0,"",COUNTIFS(F113:O113,"&gt;=0",F113:O113,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q113" s="15">
-        <f>IF(P113="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F113:O113,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F113:O113,F113:O113,"&gt;=0",F113:O113,"&lt;=20")))</f>
+        <f>IF(P113="","",SUMIFS(F113:O113,F113:O113,"&gt;=0",F113:O113,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R113" s="15">
@@ -5310,11 +5279,11 @@
       <c r="N114" s="14" t="n"/>
       <c r="O114" s="14" t="n"/>
       <c r="P114" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F114:O114,'Conversión'!$A$5:$A$8)),COUNTIFS(F114:O114,"&gt;=0",F114:O114,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F114:O114,'Conversión'!$A$5:$A$8)),COUNTIFS(F114:O114,"&gt;=0",F114:O114,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F114:O114,"&gt;=0",F114:O114,"&lt;=20")=0,"",COUNTIFS(F114:O114,"&gt;=0",F114:O114,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q114" s="15">
-        <f>IF(P114="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F114:O114,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F114:O114,F114:O114,"&gt;=0",F114:O114,"&lt;=20")))</f>
+        <f>IF(P114="","",SUMIFS(F114:O114,F114:O114,"&gt;=0",F114:O114,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R114" s="15">
@@ -5347,11 +5316,11 @@
       <c r="N115" s="14" t="n"/>
       <c r="O115" s="14" t="n"/>
       <c r="P115" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F115:O115,'Conversión'!$A$5:$A$8)),COUNTIFS(F115:O115,"&gt;=0",F115:O115,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F115:O115,'Conversión'!$A$5:$A$8)),COUNTIFS(F115:O115,"&gt;=0",F115:O115,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F115:O115,"&gt;=0",F115:O115,"&lt;=20")=0,"",COUNTIFS(F115:O115,"&gt;=0",F115:O115,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q115" s="15">
-        <f>IF(P115="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F115:O115,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F115:O115,F115:O115,"&gt;=0",F115:O115,"&lt;=20")))</f>
+        <f>IF(P115="","",SUMIFS(F115:O115,F115:O115,"&gt;=0",F115:O115,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R115" s="15">
@@ -5384,11 +5353,11 @@
       <c r="N116" s="14" t="n"/>
       <c r="O116" s="14" t="n"/>
       <c r="P116" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F116:O116,'Conversión'!$A$5:$A$8)),COUNTIFS(F116:O116,"&gt;=0",F116:O116,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F116:O116,'Conversión'!$A$5:$A$8)),COUNTIFS(F116:O116,"&gt;=0",F116:O116,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F116:O116,"&gt;=0",F116:O116,"&lt;=20")=0,"",COUNTIFS(F116:O116,"&gt;=0",F116:O116,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q116" s="15">
-        <f>IF(P116="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F116:O116,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F116:O116,F116:O116,"&gt;=0",F116:O116,"&lt;=20")))</f>
+        <f>IF(P116="","",SUMIFS(F116:O116,F116:O116,"&gt;=0",F116:O116,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R116" s="15">
@@ -5421,11 +5390,11 @@
       <c r="N117" s="14" t="n"/>
       <c r="O117" s="14" t="n"/>
       <c r="P117" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F117:O117,'Conversión'!$A$5:$A$8)),COUNTIFS(F117:O117,"&gt;=0",F117:O117,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F117:O117,'Conversión'!$A$5:$A$8)),COUNTIFS(F117:O117,"&gt;=0",F117:O117,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F117:O117,"&gt;=0",F117:O117,"&lt;=20")=0,"",COUNTIFS(F117:O117,"&gt;=0",F117:O117,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q117" s="15">
-        <f>IF(P117="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F117:O117,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F117:O117,F117:O117,"&gt;=0",F117:O117,"&lt;=20")))</f>
+        <f>IF(P117="","",SUMIFS(F117:O117,F117:O117,"&gt;=0",F117:O117,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R117" s="15">
@@ -5458,11 +5427,11 @@
       <c r="N118" s="14" t="n"/>
       <c r="O118" s="14" t="n"/>
       <c r="P118" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F118:O118,'Conversión'!$A$5:$A$8)),COUNTIFS(F118:O118,"&gt;=0",F118:O118,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F118:O118,'Conversión'!$A$5:$A$8)),COUNTIFS(F118:O118,"&gt;=0",F118:O118,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F118:O118,"&gt;=0",F118:O118,"&lt;=20")=0,"",COUNTIFS(F118:O118,"&gt;=0",F118:O118,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q118" s="15">
-        <f>IF(P118="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F118:O118,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F118:O118,F118:O118,"&gt;=0",F118:O118,"&lt;=20")))</f>
+        <f>IF(P118="","",SUMIFS(F118:O118,F118:O118,"&gt;=0",F118:O118,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R118" s="15">
@@ -5495,11 +5464,11 @@
       <c r="N119" s="14" t="n"/>
       <c r="O119" s="14" t="n"/>
       <c r="P119" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F119:O119,'Conversión'!$A$5:$A$8)),COUNTIFS(F119:O119,"&gt;=0",F119:O119,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F119:O119,'Conversión'!$A$5:$A$8)),COUNTIFS(F119:O119,"&gt;=0",F119:O119,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F119:O119,"&gt;=0",F119:O119,"&lt;=20")=0,"",COUNTIFS(F119:O119,"&gt;=0",F119:O119,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q119" s="15">
-        <f>IF(P119="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F119:O119,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F119:O119,F119:O119,"&gt;=0",F119:O119,"&lt;=20")))</f>
+        <f>IF(P119="","",SUMIFS(F119:O119,F119:O119,"&gt;=0",F119:O119,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R119" s="15">
@@ -5532,11 +5501,11 @@
       <c r="N120" s="14" t="n"/>
       <c r="O120" s="14" t="n"/>
       <c r="P120" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F120:O120,'Conversión'!$A$5:$A$8)),COUNTIFS(F120:O120,"&gt;=0",F120:O120,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F120:O120,'Conversión'!$A$5:$A$8)),COUNTIFS(F120:O120,"&gt;=0",F120:O120,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F120:O120,"&gt;=0",F120:O120,"&lt;=20")=0,"",COUNTIFS(F120:O120,"&gt;=0",F120:O120,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q120" s="15">
-        <f>IF(P120="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F120:O120,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F120:O120,F120:O120,"&gt;=0",F120:O120,"&lt;=20")))</f>
+        <f>IF(P120="","",SUMIFS(F120:O120,F120:O120,"&gt;=0",F120:O120,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R120" s="15">
@@ -5569,11 +5538,11 @@
       <c r="N121" s="14" t="n"/>
       <c r="O121" s="14" t="n"/>
       <c r="P121" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F121:O121,'Conversión'!$A$5:$A$8)),COUNTIFS(F121:O121,"&gt;=0",F121:O121,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F121:O121,'Conversión'!$A$5:$A$8)),COUNTIFS(F121:O121,"&gt;=0",F121:O121,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F121:O121,"&gt;=0",F121:O121,"&lt;=20")=0,"",COUNTIFS(F121:O121,"&gt;=0",F121:O121,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q121" s="15">
-        <f>IF(P121="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F121:O121,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F121:O121,F121:O121,"&gt;=0",F121:O121,"&lt;=20")))</f>
+        <f>IF(P121="","",SUMIFS(F121:O121,F121:O121,"&gt;=0",F121:O121,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R121" s="15">
@@ -5606,11 +5575,11 @@
       <c r="N122" s="14" t="n"/>
       <c r="O122" s="14" t="n"/>
       <c r="P122" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F122:O122,'Conversión'!$A$5:$A$8)),COUNTIFS(F122:O122,"&gt;=0",F122:O122,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F122:O122,'Conversión'!$A$5:$A$8)),COUNTIFS(F122:O122,"&gt;=0",F122:O122,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F122:O122,"&gt;=0",F122:O122,"&lt;=20")=0,"",COUNTIFS(F122:O122,"&gt;=0",F122:O122,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q122" s="15">
-        <f>IF(P122="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F122:O122,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F122:O122,F122:O122,"&gt;=0",F122:O122,"&lt;=20")))</f>
+        <f>IF(P122="","",SUMIFS(F122:O122,F122:O122,"&gt;=0",F122:O122,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R122" s="15">
@@ -5643,11 +5612,11 @@
       <c r="N123" s="14" t="n"/>
       <c r="O123" s="14" t="n"/>
       <c r="P123" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F123:O123,'Conversión'!$A$5:$A$8)),COUNTIFS(F123:O123,"&gt;=0",F123:O123,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F123:O123,'Conversión'!$A$5:$A$8)),COUNTIFS(F123:O123,"&gt;=0",F123:O123,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F123:O123,"&gt;=0",F123:O123,"&lt;=20")=0,"",COUNTIFS(F123:O123,"&gt;=0",F123:O123,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q123" s="15">
-        <f>IF(P123="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F123:O123,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F123:O123,F123:O123,"&gt;=0",F123:O123,"&lt;=20")))</f>
+        <f>IF(P123="","",SUMIFS(F123:O123,F123:O123,"&gt;=0",F123:O123,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R123" s="15">
@@ -5680,11 +5649,11 @@
       <c r="N124" s="14" t="n"/>
       <c r="O124" s="14" t="n"/>
       <c r="P124" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F124:O124,'Conversión'!$A$5:$A$8)),COUNTIFS(F124:O124,"&gt;=0",F124:O124,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F124:O124,'Conversión'!$A$5:$A$8)),COUNTIFS(F124:O124,"&gt;=0",F124:O124,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F124:O124,"&gt;=0",F124:O124,"&lt;=20")=0,"",COUNTIFS(F124:O124,"&gt;=0",F124:O124,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q124" s="15">
-        <f>IF(P124="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F124:O124,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F124:O124,F124:O124,"&gt;=0",F124:O124,"&lt;=20")))</f>
+        <f>IF(P124="","",SUMIFS(F124:O124,F124:O124,"&gt;=0",F124:O124,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R124" s="15">
@@ -5717,11 +5686,11 @@
       <c r="N125" s="14" t="n"/>
       <c r="O125" s="14" t="n"/>
       <c r="P125" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F125:O125,'Conversión'!$A$5:$A$8)),COUNTIFS(F125:O125,"&gt;=0",F125:O125,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F125:O125,'Conversión'!$A$5:$A$8)),COUNTIFS(F125:O125,"&gt;=0",F125:O125,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F125:O125,"&gt;=0",F125:O125,"&lt;=20")=0,"",COUNTIFS(F125:O125,"&gt;=0",F125:O125,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q125" s="15">
-        <f>IF(P125="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F125:O125,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F125:O125,F125:O125,"&gt;=0",F125:O125,"&lt;=20")))</f>
+        <f>IF(P125="","",SUMIFS(F125:O125,F125:O125,"&gt;=0",F125:O125,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R125" s="15">
@@ -5754,11 +5723,11 @@
       <c r="N126" s="14" t="n"/>
       <c r="O126" s="14" t="n"/>
       <c r="P126" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F126:O126,'Conversión'!$A$5:$A$8)),COUNTIFS(F126:O126,"&gt;=0",F126:O126,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F126:O126,'Conversión'!$A$5:$A$8)),COUNTIFS(F126:O126,"&gt;=0",F126:O126,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F126:O126,"&gt;=0",F126:O126,"&lt;=20")=0,"",COUNTIFS(F126:O126,"&gt;=0",F126:O126,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q126" s="15">
-        <f>IF(P126="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F126:O126,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F126:O126,F126:O126,"&gt;=0",F126:O126,"&lt;=20")))</f>
+        <f>IF(P126="","",SUMIFS(F126:O126,F126:O126,"&gt;=0",F126:O126,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R126" s="15">
@@ -5791,11 +5760,11 @@
       <c r="N127" s="14" t="n"/>
       <c r="O127" s="14" t="n"/>
       <c r="P127" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F127:O127,'Conversión'!$A$5:$A$8)),COUNTIFS(F127:O127,"&gt;=0",F127:O127,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F127:O127,'Conversión'!$A$5:$A$8)),COUNTIFS(F127:O127,"&gt;=0",F127:O127,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F127:O127,"&gt;=0",F127:O127,"&lt;=20")=0,"",COUNTIFS(F127:O127,"&gt;=0",F127:O127,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q127" s="15">
-        <f>IF(P127="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F127:O127,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F127:O127,F127:O127,"&gt;=0",F127:O127,"&lt;=20")))</f>
+        <f>IF(P127="","",SUMIFS(F127:O127,F127:O127,"&gt;=0",F127:O127,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R127" s="15">
@@ -5828,11 +5797,11 @@
       <c r="N128" s="14" t="n"/>
       <c r="O128" s="14" t="n"/>
       <c r="P128" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F128:O128,'Conversión'!$A$5:$A$8)),COUNTIFS(F128:O128,"&gt;=0",F128:O128,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F128:O128,'Conversión'!$A$5:$A$8)),COUNTIFS(F128:O128,"&gt;=0",F128:O128,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F128:O128,"&gt;=0",F128:O128,"&lt;=20")=0,"",COUNTIFS(F128:O128,"&gt;=0",F128:O128,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q128" s="15">
-        <f>IF(P128="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F128:O128,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F128:O128,F128:O128,"&gt;=0",F128:O128,"&lt;=20")))</f>
+        <f>IF(P128="","",SUMIFS(F128:O128,F128:O128,"&gt;=0",F128:O128,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R128" s="15">
@@ -5865,11 +5834,11 @@
       <c r="N129" s="14" t="n"/>
       <c r="O129" s="14" t="n"/>
       <c r="P129" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F129:O129,'Conversión'!$A$5:$A$8)),COUNTIFS(F129:O129,"&gt;=0",F129:O129,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F129:O129,'Conversión'!$A$5:$A$8)),COUNTIFS(F129:O129,"&gt;=0",F129:O129,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F129:O129,"&gt;=0",F129:O129,"&lt;=20")=0,"",COUNTIFS(F129:O129,"&gt;=0",F129:O129,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q129" s="15">
-        <f>IF(P129="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F129:O129,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F129:O129,F129:O129,"&gt;=0",F129:O129,"&lt;=20")))</f>
+        <f>IF(P129="","",SUMIFS(F129:O129,F129:O129,"&gt;=0",F129:O129,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R129" s="15">
@@ -5902,11 +5871,11 @@
       <c r="N130" s="14" t="n"/>
       <c r="O130" s="14" t="n"/>
       <c r="P130" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F130:O130,'Conversión'!$A$5:$A$8)),COUNTIFS(F130:O130,"&gt;=0",F130:O130,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F130:O130,'Conversión'!$A$5:$A$8)),COUNTIFS(F130:O130,"&gt;=0",F130:O130,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F130:O130,"&gt;=0",F130:O130,"&lt;=20")=0,"",COUNTIFS(F130:O130,"&gt;=0",F130:O130,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q130" s="15">
-        <f>IF(P130="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F130:O130,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F130:O130,F130:O130,"&gt;=0",F130:O130,"&lt;=20")))</f>
+        <f>IF(P130="","",SUMIFS(F130:O130,F130:O130,"&gt;=0",F130:O130,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R130" s="15">
@@ -5939,11 +5908,11 @@
       <c r="N131" s="14" t="n"/>
       <c r="O131" s="14" t="n"/>
       <c r="P131" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F131:O131,'Conversión'!$A$5:$A$8)),COUNTIFS(F131:O131,"&gt;=0",F131:O131,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F131:O131,'Conversión'!$A$5:$A$8)),COUNTIFS(F131:O131,"&gt;=0",F131:O131,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F131:O131,"&gt;=0",F131:O131,"&lt;=20")=0,"",COUNTIFS(F131:O131,"&gt;=0",F131:O131,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q131" s="15">
-        <f>IF(P131="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F131:O131,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F131:O131,F131:O131,"&gt;=0",F131:O131,"&lt;=20")))</f>
+        <f>IF(P131="","",SUMIFS(F131:O131,F131:O131,"&gt;=0",F131:O131,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R131" s="15">
@@ -5976,11 +5945,11 @@
       <c r="N132" s="14" t="n"/>
       <c r="O132" s="14" t="n"/>
       <c r="P132" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F132:O132,'Conversión'!$A$5:$A$8)),COUNTIFS(F132:O132,"&gt;=0",F132:O132,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F132:O132,'Conversión'!$A$5:$A$8)),COUNTIFS(F132:O132,"&gt;=0",F132:O132,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F132:O132,"&gt;=0",F132:O132,"&lt;=20")=0,"",COUNTIFS(F132:O132,"&gt;=0",F132:O132,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q132" s="15">
-        <f>IF(P132="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F132:O132,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F132:O132,F132:O132,"&gt;=0",F132:O132,"&lt;=20")))</f>
+        <f>IF(P132="","",SUMIFS(F132:O132,F132:O132,"&gt;=0",F132:O132,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R132" s="15">
@@ -6013,11 +5982,11 @@
       <c r="N133" s="14" t="n"/>
       <c r="O133" s="14" t="n"/>
       <c r="P133" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F133:O133,'Conversión'!$A$5:$A$8)),COUNTIFS(F133:O133,"&gt;=0",F133:O133,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F133:O133,'Conversión'!$A$5:$A$8)),COUNTIFS(F133:O133,"&gt;=0",F133:O133,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F133:O133,"&gt;=0",F133:O133,"&lt;=20")=0,"",COUNTIFS(F133:O133,"&gt;=0",F133:O133,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q133" s="15">
-        <f>IF(P133="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F133:O133,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F133:O133,F133:O133,"&gt;=0",F133:O133,"&lt;=20")))</f>
+        <f>IF(P133="","",SUMIFS(F133:O133,F133:O133,"&gt;=0",F133:O133,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R133" s="15">
@@ -6050,11 +6019,11 @@
       <c r="N134" s="14" t="n"/>
       <c r="O134" s="14" t="n"/>
       <c r="P134" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F134:O134,'Conversión'!$A$5:$A$8)),COUNTIFS(F134:O134,"&gt;=0",F134:O134,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F134:O134,'Conversión'!$A$5:$A$8)),COUNTIFS(F134:O134,"&gt;=0",F134:O134,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F134:O134,"&gt;=0",F134:O134,"&lt;=20")=0,"",COUNTIFS(F134:O134,"&gt;=0",F134:O134,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q134" s="15">
-        <f>IF(P134="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F134:O134,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F134:O134,F134:O134,"&gt;=0",F134:O134,"&lt;=20")))</f>
+        <f>IF(P134="","",SUMIFS(F134:O134,F134:O134,"&gt;=0",F134:O134,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R134" s="15">
@@ -6087,11 +6056,11 @@
       <c r="N135" s="14" t="n"/>
       <c r="O135" s="14" t="n"/>
       <c r="P135" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F135:O135,'Conversión'!$A$5:$A$8)),COUNTIFS(F135:O135,"&gt;=0",F135:O135,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F135:O135,'Conversión'!$A$5:$A$8)),COUNTIFS(F135:O135,"&gt;=0",F135:O135,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F135:O135,"&gt;=0",F135:O135,"&lt;=20")=0,"",COUNTIFS(F135:O135,"&gt;=0",F135:O135,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q135" s="15">
-        <f>IF(P135="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F135:O135,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F135:O135,F135:O135,"&gt;=0",F135:O135,"&lt;=20")))</f>
+        <f>IF(P135="","",SUMIFS(F135:O135,F135:O135,"&gt;=0",F135:O135,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R135" s="15">
@@ -6124,11 +6093,11 @@
       <c r="N136" s="14" t="n"/>
       <c r="O136" s="14" t="n"/>
       <c r="P136" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F136:O136,'Conversión'!$A$5:$A$8)),COUNTIFS(F136:O136,"&gt;=0",F136:O136,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F136:O136,'Conversión'!$A$5:$A$8)),COUNTIFS(F136:O136,"&gt;=0",F136:O136,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F136:O136,"&gt;=0",F136:O136,"&lt;=20")=0,"",COUNTIFS(F136:O136,"&gt;=0",F136:O136,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q136" s="15">
-        <f>IF(P136="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F136:O136,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F136:O136,F136:O136,"&gt;=0",F136:O136,"&lt;=20")))</f>
+        <f>IF(P136="","",SUMIFS(F136:O136,F136:O136,"&gt;=0",F136:O136,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R136" s="15">
@@ -6161,11 +6130,11 @@
       <c r="N137" s="14" t="n"/>
       <c r="O137" s="14" t="n"/>
       <c r="P137" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F137:O137,'Conversión'!$A$5:$A$8)),COUNTIFS(F137:O137,"&gt;=0",F137:O137,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F137:O137,'Conversión'!$A$5:$A$8)),COUNTIFS(F137:O137,"&gt;=0",F137:O137,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F137:O137,"&gt;=0",F137:O137,"&lt;=20")=0,"",COUNTIFS(F137:O137,"&gt;=0",F137:O137,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q137" s="15">
-        <f>IF(P137="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F137:O137,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F137:O137,F137:O137,"&gt;=0",F137:O137,"&lt;=20")))</f>
+        <f>IF(P137="","",SUMIFS(F137:O137,F137:O137,"&gt;=0",F137:O137,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R137" s="15">
@@ -6198,11 +6167,11 @@
       <c r="N138" s="14" t="n"/>
       <c r="O138" s="14" t="n"/>
       <c r="P138" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F138:O138,'Conversión'!$A$5:$A$8)),COUNTIFS(F138:O138,"&gt;=0",F138:O138,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F138:O138,'Conversión'!$A$5:$A$8)),COUNTIFS(F138:O138,"&gt;=0",F138:O138,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F138:O138,"&gt;=0",F138:O138,"&lt;=20")=0,"",COUNTIFS(F138:O138,"&gt;=0",F138:O138,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q138" s="15">
-        <f>IF(P138="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F138:O138,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F138:O138,F138:O138,"&gt;=0",F138:O138,"&lt;=20")))</f>
+        <f>IF(P138="","",SUMIFS(F138:O138,F138:O138,"&gt;=0",F138:O138,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R138" s="15">
@@ -6235,11 +6204,11 @@
       <c r="N139" s="14" t="n"/>
       <c r="O139" s="14" t="n"/>
       <c r="P139" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F139:O139,'Conversión'!$A$5:$A$8)),COUNTIFS(F139:O139,"&gt;=0",F139:O139,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F139:O139,'Conversión'!$A$5:$A$8)),COUNTIFS(F139:O139,"&gt;=0",F139:O139,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F139:O139,"&gt;=0",F139:O139,"&lt;=20")=0,"",COUNTIFS(F139:O139,"&gt;=0",F139:O139,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q139" s="15">
-        <f>IF(P139="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F139:O139,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F139:O139,F139:O139,"&gt;=0",F139:O139,"&lt;=20")))</f>
+        <f>IF(P139="","",SUMIFS(F139:O139,F139:O139,"&gt;=0",F139:O139,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R139" s="15">
@@ -6272,11 +6241,11 @@
       <c r="N140" s="14" t="n"/>
       <c r="O140" s="14" t="n"/>
       <c r="P140" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F140:O140,'Conversión'!$A$5:$A$8)),COUNTIFS(F140:O140,"&gt;=0",F140:O140,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F140:O140,'Conversión'!$A$5:$A$8)),COUNTIFS(F140:O140,"&gt;=0",F140:O140,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F140:O140,"&gt;=0",F140:O140,"&lt;=20")=0,"",COUNTIFS(F140:O140,"&gt;=0",F140:O140,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q140" s="15">
-        <f>IF(P140="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F140:O140,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F140:O140,F140:O140,"&gt;=0",F140:O140,"&lt;=20")))</f>
+        <f>IF(P140="","",SUMIFS(F140:O140,F140:O140,"&gt;=0",F140:O140,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R140" s="15">
@@ -6309,11 +6278,11 @@
       <c r="N141" s="14" t="n"/>
       <c r="O141" s="14" t="n"/>
       <c r="P141" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F141:O141,'Conversión'!$A$5:$A$8)),COUNTIFS(F141:O141,"&gt;=0",F141:O141,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F141:O141,'Conversión'!$A$5:$A$8)),COUNTIFS(F141:O141,"&gt;=0",F141:O141,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F141:O141,"&gt;=0",F141:O141,"&lt;=20")=0,"",COUNTIFS(F141:O141,"&gt;=0",F141:O141,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q141" s="15">
-        <f>IF(P141="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F141:O141,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F141:O141,F141:O141,"&gt;=0",F141:O141,"&lt;=20")))</f>
+        <f>IF(P141="","",SUMIFS(F141:O141,F141:O141,"&gt;=0",F141:O141,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R141" s="15">
@@ -6346,11 +6315,11 @@
       <c r="N142" s="14" t="n"/>
       <c r="O142" s="14" t="n"/>
       <c r="P142" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F142:O142,'Conversión'!$A$5:$A$8)),COUNTIFS(F142:O142,"&gt;=0",F142:O142,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F142:O142,'Conversión'!$A$5:$A$8)),COUNTIFS(F142:O142,"&gt;=0",F142:O142,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F142:O142,"&gt;=0",F142:O142,"&lt;=20")=0,"",COUNTIFS(F142:O142,"&gt;=0",F142:O142,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q142" s="15">
-        <f>IF(P142="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F142:O142,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F142:O142,F142:O142,"&gt;=0",F142:O142,"&lt;=20")))</f>
+        <f>IF(P142="","",SUMIFS(F142:O142,F142:O142,"&gt;=0",F142:O142,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R142" s="15">
@@ -6383,11 +6352,11 @@
       <c r="N143" s="14" t="n"/>
       <c r="O143" s="14" t="n"/>
       <c r="P143" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F143:O143,'Conversión'!$A$5:$A$8)),COUNTIFS(F143:O143,"&gt;=0",F143:O143,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F143:O143,'Conversión'!$A$5:$A$8)),COUNTIFS(F143:O143,"&gt;=0",F143:O143,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F143:O143,"&gt;=0",F143:O143,"&lt;=20")=0,"",COUNTIFS(F143:O143,"&gt;=0",F143:O143,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q143" s="15">
-        <f>IF(P143="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F143:O143,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F143:O143,F143:O143,"&gt;=0",F143:O143,"&lt;=20")))</f>
+        <f>IF(P143="","",SUMIFS(F143:O143,F143:O143,"&gt;=0",F143:O143,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R143" s="15">
@@ -6420,11 +6389,11 @@
       <c r="N144" s="14" t="n"/>
       <c r="O144" s="14" t="n"/>
       <c r="P144" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F144:O144,'Conversión'!$A$5:$A$8)),COUNTIFS(F144:O144,"&gt;=0",F144:O144,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F144:O144,'Conversión'!$A$5:$A$8)),COUNTIFS(F144:O144,"&gt;=0",F144:O144,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F144:O144,"&gt;=0",F144:O144,"&lt;=20")=0,"",COUNTIFS(F144:O144,"&gt;=0",F144:O144,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q144" s="15">
-        <f>IF(P144="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F144:O144,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F144:O144,F144:O144,"&gt;=0",F144:O144,"&lt;=20")))</f>
+        <f>IF(P144="","",SUMIFS(F144:O144,F144:O144,"&gt;=0",F144:O144,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R144" s="15">
@@ -6457,11 +6426,11 @@
       <c r="N145" s="14" t="n"/>
       <c r="O145" s="14" t="n"/>
       <c r="P145" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F145:O145,'Conversión'!$A$5:$A$8)),COUNTIFS(F145:O145,"&gt;=0",F145:O145,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F145:O145,'Conversión'!$A$5:$A$8)),COUNTIFS(F145:O145,"&gt;=0",F145:O145,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F145:O145,"&gt;=0",F145:O145,"&lt;=20")=0,"",COUNTIFS(F145:O145,"&gt;=0",F145:O145,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q145" s="15">
-        <f>IF(P145="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F145:O145,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F145:O145,F145:O145,"&gt;=0",F145:O145,"&lt;=20")))</f>
+        <f>IF(P145="","",SUMIFS(F145:O145,F145:O145,"&gt;=0",F145:O145,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R145" s="15">
@@ -6494,11 +6463,11 @@
       <c r="N146" s="14" t="n"/>
       <c r="O146" s="14" t="n"/>
       <c r="P146" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F146:O146,'Conversión'!$A$5:$A$8)),COUNTIFS(F146:O146,"&gt;=0",F146:O146,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F146:O146,'Conversión'!$A$5:$A$8)),COUNTIFS(F146:O146,"&gt;=0",F146:O146,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F146:O146,"&gt;=0",F146:O146,"&lt;=20")=0,"",COUNTIFS(F146:O146,"&gt;=0",F146:O146,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q146" s="15">
-        <f>IF(P146="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F146:O146,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F146:O146,F146:O146,"&gt;=0",F146:O146,"&lt;=20")))</f>
+        <f>IF(P146="","",SUMIFS(F146:O146,F146:O146,"&gt;=0",F146:O146,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R146" s="15">
@@ -6531,11 +6500,11 @@
       <c r="N147" s="14" t="n"/>
       <c r="O147" s="14" t="n"/>
       <c r="P147" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F147:O147,'Conversión'!$A$5:$A$8)),COUNTIFS(F147:O147,"&gt;=0",F147:O147,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F147:O147,'Conversión'!$A$5:$A$8)),COUNTIFS(F147:O147,"&gt;=0",F147:O147,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F147:O147,"&gt;=0",F147:O147,"&lt;=20")=0,"",COUNTIFS(F147:O147,"&gt;=0",F147:O147,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q147" s="15">
-        <f>IF(P147="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F147:O147,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F147:O147,F147:O147,"&gt;=0",F147:O147,"&lt;=20")))</f>
+        <f>IF(P147="","",SUMIFS(F147:O147,F147:O147,"&gt;=0",F147:O147,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R147" s="15">
@@ -6568,11 +6537,11 @@
       <c r="N148" s="14" t="n"/>
       <c r="O148" s="14" t="n"/>
       <c r="P148" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F148:O148,'Conversión'!$A$5:$A$8)),COUNTIFS(F148:O148,"&gt;=0",F148:O148,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F148:O148,'Conversión'!$A$5:$A$8)),COUNTIFS(F148:O148,"&gt;=0",F148:O148,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F148:O148,"&gt;=0",F148:O148,"&lt;=20")=0,"",COUNTIFS(F148:O148,"&gt;=0",F148:O148,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q148" s="15">
-        <f>IF(P148="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F148:O148,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F148:O148,F148:O148,"&gt;=0",F148:O148,"&lt;=20")))</f>
+        <f>IF(P148="","",SUMIFS(F148:O148,F148:O148,"&gt;=0",F148:O148,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R148" s="15">
@@ -6605,11 +6574,11 @@
       <c r="N149" s="14" t="n"/>
       <c r="O149" s="14" t="n"/>
       <c r="P149" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F149:O149,'Conversión'!$A$5:$A$8)),COUNTIFS(F149:O149,"&gt;=0",F149:O149,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F149:O149,'Conversión'!$A$5:$A$8)),COUNTIFS(F149:O149,"&gt;=0",F149:O149,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F149:O149,"&gt;=0",F149:O149,"&lt;=20")=0,"",COUNTIFS(F149:O149,"&gt;=0",F149:O149,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q149" s="15">
-        <f>IF(P149="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F149:O149,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F149:O149,F149:O149,"&gt;=0",F149:O149,"&lt;=20")))</f>
+        <f>IF(P149="","",SUMIFS(F149:O149,F149:O149,"&gt;=0",F149:O149,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R149" s="15">
@@ -6642,11 +6611,11 @@
       <c r="N150" s="14" t="n"/>
       <c r="O150" s="14" t="n"/>
       <c r="P150" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F150:O150,'Conversión'!$A$5:$A$8)),COUNTIFS(F150:O150,"&gt;=0",F150:O150,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F150:O150,'Conversión'!$A$5:$A$8)),COUNTIFS(F150:O150,"&gt;=0",F150:O150,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F150:O150,"&gt;=0",F150:O150,"&lt;=20")=0,"",COUNTIFS(F150:O150,"&gt;=0",F150:O150,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q150" s="15">
-        <f>IF(P150="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F150:O150,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F150:O150,F150:O150,"&gt;=0",F150:O150,"&lt;=20")))</f>
+        <f>IF(P150="","",SUMIFS(F150:O150,F150:O150,"&gt;=0",F150:O150,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R150" s="15">
@@ -6679,11 +6648,11 @@
       <c r="N151" s="14" t="n"/>
       <c r="O151" s="14" t="n"/>
       <c r="P151" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F151:O151,'Conversión'!$A$5:$A$8)),COUNTIFS(F151:O151,"&gt;=0",F151:O151,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F151:O151,'Conversión'!$A$5:$A$8)),COUNTIFS(F151:O151,"&gt;=0",F151:O151,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F151:O151,"&gt;=0",F151:O151,"&lt;=20")=0,"",COUNTIFS(F151:O151,"&gt;=0",F151:O151,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q151" s="15">
-        <f>IF(P151="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F151:O151,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F151:O151,F151:O151,"&gt;=0",F151:O151,"&lt;=20")))</f>
+        <f>IF(P151="","",SUMIFS(F151:O151,F151:O151,"&gt;=0",F151:O151,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R151" s="15">
@@ -6716,11 +6685,11 @@
       <c r="N152" s="14" t="n"/>
       <c r="O152" s="14" t="n"/>
       <c r="P152" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F152:O152,'Conversión'!$A$5:$A$8)),COUNTIFS(F152:O152,"&gt;=0",F152:O152,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F152:O152,'Conversión'!$A$5:$A$8)),COUNTIFS(F152:O152,"&gt;=0",F152:O152,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F152:O152,"&gt;=0",F152:O152,"&lt;=20")=0,"",COUNTIFS(F152:O152,"&gt;=0",F152:O152,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q152" s="15">
-        <f>IF(P152="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F152:O152,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F152:O152,F152:O152,"&gt;=0",F152:O152,"&lt;=20")))</f>
+        <f>IF(P152="","",SUMIFS(F152:O152,F152:O152,"&gt;=0",F152:O152,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R152" s="15">
@@ -6753,11 +6722,11 @@
       <c r="N153" s="14" t="n"/>
       <c r="O153" s="14" t="n"/>
       <c r="P153" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F153:O153,'Conversión'!$A$5:$A$8)),COUNTIFS(F153:O153,"&gt;=0",F153:O153,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F153:O153,'Conversión'!$A$5:$A$8)),COUNTIFS(F153:O153,"&gt;=0",F153:O153,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F153:O153,"&gt;=0",F153:O153,"&lt;=20")=0,"",COUNTIFS(F153:O153,"&gt;=0",F153:O153,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q153" s="15">
-        <f>IF(P153="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F153:O153,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F153:O153,F153:O153,"&gt;=0",F153:O153,"&lt;=20")))</f>
+        <f>IF(P153="","",SUMIFS(F153:O153,F153:O153,"&gt;=0",F153:O153,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R153" s="15">
@@ -6790,11 +6759,11 @@
       <c r="N154" s="14" t="n"/>
       <c r="O154" s="14" t="n"/>
       <c r="P154" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F154:O154,'Conversión'!$A$5:$A$8)),COUNTIFS(F154:O154,"&gt;=0",F154:O154,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F154:O154,'Conversión'!$A$5:$A$8)),COUNTIFS(F154:O154,"&gt;=0",F154:O154,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F154:O154,"&gt;=0",F154:O154,"&lt;=20")=0,"",COUNTIFS(F154:O154,"&gt;=0",F154:O154,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q154" s="15">
-        <f>IF(P154="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F154:O154,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F154:O154,F154:O154,"&gt;=0",F154:O154,"&lt;=20")))</f>
+        <f>IF(P154="","",SUMIFS(F154:O154,F154:O154,"&gt;=0",F154:O154,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R154" s="15">
@@ -6827,11 +6796,11 @@
       <c r="N155" s="14" t="n"/>
       <c r="O155" s="14" t="n"/>
       <c r="P155" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F155:O155,'Conversión'!$A$5:$A$8)),COUNTIFS(F155:O155,"&gt;=0",F155:O155,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F155:O155,'Conversión'!$A$5:$A$8)),COUNTIFS(F155:O155,"&gt;=0",F155:O155,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F155:O155,"&gt;=0",F155:O155,"&lt;=20")=0,"",COUNTIFS(F155:O155,"&gt;=0",F155:O155,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q155" s="15">
-        <f>IF(P155="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F155:O155,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F155:O155,F155:O155,"&gt;=0",F155:O155,"&lt;=20")))</f>
+        <f>IF(P155="","",SUMIFS(F155:O155,F155:O155,"&gt;=0",F155:O155,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R155" s="15">
@@ -6864,11 +6833,11 @@
       <c r="N156" s="14" t="n"/>
       <c r="O156" s="14" t="n"/>
       <c r="P156" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F156:O156,'Conversión'!$A$5:$A$8)),COUNTIFS(F156:O156,"&gt;=0",F156:O156,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F156:O156,'Conversión'!$A$5:$A$8)),COUNTIFS(F156:O156,"&gt;=0",F156:O156,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F156:O156,"&gt;=0",F156:O156,"&lt;=20")=0,"",COUNTIFS(F156:O156,"&gt;=0",F156:O156,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q156" s="15">
-        <f>IF(P156="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F156:O156,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F156:O156,F156:O156,"&gt;=0",F156:O156,"&lt;=20")))</f>
+        <f>IF(P156="","",SUMIFS(F156:O156,F156:O156,"&gt;=0",F156:O156,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R156" s="15">
@@ -6901,11 +6870,11 @@
       <c r="N157" s="14" t="n"/>
       <c r="O157" s="14" t="n"/>
       <c r="P157" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F157:O157,'Conversión'!$A$5:$A$8)),COUNTIFS(F157:O157,"&gt;=0",F157:O157,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F157:O157,'Conversión'!$A$5:$A$8)),COUNTIFS(F157:O157,"&gt;=0",F157:O157,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F157:O157,"&gt;=0",F157:O157,"&lt;=20")=0,"",COUNTIFS(F157:O157,"&gt;=0",F157:O157,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q157" s="15">
-        <f>IF(P157="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F157:O157,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F157:O157,F157:O157,"&gt;=0",F157:O157,"&lt;=20")))</f>
+        <f>IF(P157="","",SUMIFS(F157:O157,F157:O157,"&gt;=0",F157:O157,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R157" s="15">
@@ -6938,11 +6907,11 @@
       <c r="N158" s="14" t="n"/>
       <c r="O158" s="14" t="n"/>
       <c r="P158" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F158:O158,'Conversión'!$A$5:$A$8)),COUNTIFS(F158:O158,"&gt;=0",F158:O158,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F158:O158,'Conversión'!$A$5:$A$8)),COUNTIFS(F158:O158,"&gt;=0",F158:O158,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F158:O158,"&gt;=0",F158:O158,"&lt;=20")=0,"",COUNTIFS(F158:O158,"&gt;=0",F158:O158,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q158" s="15">
-        <f>IF(P158="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F158:O158,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F158:O158,F158:O158,"&gt;=0",F158:O158,"&lt;=20")))</f>
+        <f>IF(P158="","",SUMIFS(F158:O158,F158:O158,"&gt;=0",F158:O158,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R158" s="15">
@@ -6975,11 +6944,11 @@
       <c r="N159" s="14" t="n"/>
       <c r="O159" s="14" t="n"/>
       <c r="P159" s="15">
-        <f>IF(IF($B$7="literal",SUMPRODUCT(COUNTIF(F159:O159,'Conversión'!$A$5:$A$8)),COUNTIFS(F159:O159,"&gt;=0",F159:O159,"&lt;=20"))=0,"",IF($B$7="literal",SUMPRODUCT(COUNTIF(F159:O159,'Conversión'!$A$5:$A$8)),COUNTIFS(F159:O159,"&gt;=0",F159:O159,"&lt;=20")))</f>
+        <f>IF(COUNTIFS(F159:O159,"&gt;=0",F159:O159,"&lt;=20")=0,"",COUNTIFS(F159:O159,"&gt;=0",F159:O159,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="Q159" s="15">
-        <f>IF(P159="","",IF($B$7="literal",SUMPRODUCT(COUNTIF(F159:O159,'Conversión'!$A$5:$A$8)*'Conversión'!$B$5:$B$8),SUMIFS(F159:O159,F159:O159,"&gt;=0",F159:O159,"&lt;=20")))</f>
+        <f>IF(P159="","",SUMIFS(F159:O159,F159:O159,"&gt;=0",F159:O159,"&lt;=20"))</f>
         <v/>
       </c>
       <c r="R159" s="15">
@@ -7027,64 +6996,61 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F10:F159">
     <cfRule type="expression" priority="7" dxfId="1">
-      <formula>AND(F10&lt;&gt;"",NOT(IF($B$7="literal",OR(F10="AD",F10="A",F10="B",F10="C"),AND(ISNUMBER(F10),F10&gt;=0,F10&lt;=20))))</formula>
+      <formula>AND(F10&lt;&gt;"",NOT(AND(ISNUMBER(F10),F10&gt;=0,F10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G10:G159">
     <cfRule type="expression" priority="8" dxfId="1">
-      <formula>AND(G10&lt;&gt;"",NOT(IF($B$7="literal",OR(G10="AD",G10="A",G10="B",G10="C"),AND(ISNUMBER(G10),G10&gt;=0,G10&lt;=20))))</formula>
+      <formula>AND(G10&lt;&gt;"",NOT(AND(ISNUMBER(G10),G10&gt;=0,G10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H159">
     <cfRule type="expression" priority="9" dxfId="1">
-      <formula>AND(H10&lt;&gt;"",NOT(IF($B$7="literal",OR(H10="AD",H10="A",H10="B",H10="C"),AND(ISNUMBER(H10),H10&gt;=0,H10&lt;=20))))</formula>
+      <formula>AND(H10&lt;&gt;"",NOT(AND(ISNUMBER(H10),H10&gt;=0,H10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:I159">
     <cfRule type="expression" priority="10" dxfId="1">
-      <formula>AND(I10&lt;&gt;"",NOT(IF($B$7="literal",OR(I10="AD",I10="A",I10="B",I10="C"),AND(ISNUMBER(I10),I10&gt;=0,I10&lt;=20))))</formula>
+      <formula>AND(I10&lt;&gt;"",NOT(AND(ISNUMBER(I10),I10&gt;=0,I10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J10:J159">
     <cfRule type="expression" priority="11" dxfId="1">
-      <formula>AND(J10&lt;&gt;"",NOT(IF($B$7="literal",OR(J10="AD",J10="A",J10="B",J10="C"),AND(ISNUMBER(J10),J10&gt;=0,J10&lt;=20))))</formula>
+      <formula>AND(J10&lt;&gt;"",NOT(AND(ISNUMBER(J10),J10&gt;=0,J10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K10:K159">
     <cfRule type="expression" priority="12" dxfId="1">
-      <formula>AND(K10&lt;&gt;"",NOT(IF($B$7="literal",OR(K10="AD",K10="A",K10="B",K10="C"),AND(ISNUMBER(K10),K10&gt;=0,K10&lt;=20))))</formula>
+      <formula>AND(K10&lt;&gt;"",NOT(AND(ISNUMBER(K10),K10&gt;=0,K10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L10:L159">
     <cfRule type="expression" priority="13" dxfId="1">
-      <formula>AND(L10&lt;&gt;"",NOT(IF($B$7="literal",OR(L10="AD",L10="A",L10="B",L10="C"),AND(ISNUMBER(L10),L10&gt;=0,L10&lt;=20))))</formula>
+      <formula>AND(L10&lt;&gt;"",NOT(AND(ISNUMBER(L10),L10&gt;=0,L10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M10:M159">
     <cfRule type="expression" priority="14" dxfId="1">
-      <formula>AND(M10&lt;&gt;"",NOT(IF($B$7="literal",OR(M10="AD",M10="A",M10="B",M10="C"),AND(ISNUMBER(M10),M10&gt;=0,M10&lt;=20))))</formula>
+      <formula>AND(M10&lt;&gt;"",NOT(AND(ISNUMBER(M10),M10&gt;=0,M10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N10:N159">
     <cfRule type="expression" priority="15" dxfId="1">
-      <formula>AND(N10&lt;&gt;"",NOT(IF($B$7="literal",OR(N10="AD",N10="A",N10="B",N10="C"),AND(ISNUMBER(N10),N10&gt;=0,N10&lt;=20))))</formula>
+      <formula>AND(N10&lt;&gt;"",NOT(AND(ISNUMBER(N10),N10&gt;=0,N10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O10:O159">
     <cfRule type="expression" priority="16" dxfId="1">
-      <formula>AND(O10&lt;&gt;"",NOT(IF($B$7="literal",OR(O10="AD",O10="A",O10="B",O10="C"),AND(ISNUMBER(O10),O10&gt;=0,O10&lt;=20))))</formula>
+      <formula>AND(O10&lt;&gt;"",NOT(AND(ISNUMBER(O10),O10&gt;=0,O10&lt;=20)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="21">
+  <dataValidations count="20">
     <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Año entre 2024 y 2026." type="whole" operator="between">
       <formula1>2024</formula1>
       <formula2>2026</formula2>
     </dataValidation>
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="El corte es el I bimestre." type="list">
       <formula1>"I bimestre"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una." type="list">
-      <formula1>"vigesimal,literal"</formula1>
     </dataValidation>
     <dataValidation sqref="A10:A159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Use el formato EST-001 (sin nombres ni DNI)." type="custom">
       <formula1>AND(LEN(A10)=7,LEFT(A10,4)="EST-",ISNUMBER(VALUE(RIGHT(A10,3))))</formula1>
@@ -7100,35 +7066,45 @@
     <dataValidation sqref="E10:E159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija pre o post." type="list">
       <formula1>"pre,post"</formula1>
     </dataValidation>
-    <dataValidation sqref="F10:F159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(F10="AD",F10="A",F10="B",F10="C"),AND(ISNUMBER(F10),F10&gt;=0,F10&lt;=20))</formula1>
+    <dataValidation sqref="F10:F159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="G10:G159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(G10="AD",G10="A",G10="B",G10="C"),AND(ISNUMBER(G10),G10&gt;=0,G10&lt;=20))</formula1>
+    <dataValidation sqref="G10:G159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="H10:H159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(H10="AD",H10="A",H10="B",H10="C"),AND(ISNUMBER(H10),H10&gt;=0,H10&lt;=20))</formula1>
+    <dataValidation sqref="H10:H159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="I10:I159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(I10="AD",I10="A",I10="B",I10="C"),AND(ISNUMBER(I10),I10&gt;=0,I10&lt;=20))</formula1>
+    <dataValidation sqref="I10:I159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="J10:J159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(J10="AD",J10="A",J10="B",J10="C"),AND(ISNUMBER(J10),J10&gt;=0,J10&lt;=20))</formula1>
+    <dataValidation sqref="J10:J159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="K10:K159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(K10="AD",K10="A",K10="B",K10="C"),AND(ISNUMBER(K10),K10&gt;=0,K10&lt;=20))</formula1>
+    <dataValidation sqref="K10:K159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="L10:L159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(L10="AD",L10="A",L10="B",L10="C"),AND(ISNUMBER(L10),L10&gt;=0,L10&lt;=20))</formula1>
+    <dataValidation sqref="L10:L159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="M10:M159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(M10="AD",M10="A",M10="B",M10="C"),AND(ISNUMBER(M10),M10&gt;=0,M10&lt;=20))</formula1>
+    <dataValidation sqref="M10:M159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="N10:N159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(N10="AD",N10="A",N10="B",N10="C"),AND(ISNUMBER(N10),N10&gt;=0,N10&lt;=20))</formula1>
+    <dataValidation sqref="N10:N159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="O10:O159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Vigesimal: número de 0 a 20. Literal: AD, A, B o C." type="custom">
-      <formula1>IF($B$7="literal",OR(O10="AD",O10="A",O10="B",O10="C"),AND(ISNUMBER(O10),O10&gt;=0,O10&lt;=20))</formula1>
+    <dataValidation sqref="O10:O159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La nota debe ser un número de 0 a 20." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
     <dataValidation sqref="S10:S159" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="El año debe estar entre 2024 y 2026." type="whole" operator="between">
       <formula1>2024</formula1>
@@ -7148,114 +7124,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Conversión de escala literal a numérica</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>PROVISIONAL (decisión D1): se confirma con la IE y se justifica en la tesis. Escala literal de EBR según RVM N.° 094-2020-MINEDU.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Literal</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AD</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Logro destacado</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Logro esperado</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>En inicio</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>